<commit_message>
Instruction v1.12, eight v1.11 Opus workbooks, review, cockpit, DeepSeek provider, instruction comparison
v1.12: seven general edits to v1.11 after the eight-deal review (DECISIONS_v1.12.md).
Runner: deepseek provider via OpenCode, --instruction option, usage and library versions recorded.
Checker 1.5: inferred-exit and exact-day cross-column checks.
Comparison of v1.11, v1.12 and v1.12.1 on DeepSeek flash and Opus: _dev/reviews/2026-09-21/instruction_comparison.md.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extraction/mac-gray.xlsx
+++ b/extraction/mac-gray.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal facts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rounds'!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal facts'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal facts'!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,9 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
+    <numFmt numFmtId="166" formatCode="$0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -71,7 +72,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -439,28 +440,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V50"/>
+  <dimension ref="A1:V53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
     <col width="55" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
@@ -584,7 +585,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10/23/2012</t>
+          <t>04/05/2013</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -614,24 +615,24 @@
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Target's financial adviser, hired for Mac-Gray's possible purchase of CSC (2011-2012 Discussions), not for a sale. On 04/05/2013 the board had it explore opportunities, including with Party A.</t>
+          <t>Mac-Gray's financial adviser, first seen acting in the sale context: Board authorized management to work with it to explore transactions, incl. with Party A. Engaged 10/23/2012 for the 2011–2012 Discussions (Mac-Gray's possible purchase of CSC).</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>“In connection with Mac-Gray's consideration of a possible acquisition of CSC, which we refer to as the 2011-2012 Discussions, Mac-Gray engaged BofA Merrill Lynch on October 23, 2012.” (p. 27)</t>
+          <t>“authorized Mac-Gray management to work with BofA Merrill Lynch to explore transactional opportunities that might be available to Mac-Gray” (p. 27)</t>
         </is>
       </c>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="3" t="n">
-        <v>41205</v>
+        <v>41369</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>41205</v>
+        <v>41369</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>41205</v>
+        <v>41369</v>
       </c>
     </row>
     <row r="3">
@@ -676,12 +677,12 @@
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Board authorized this on 04/05 as part of exploring opportunities. Party A said it might consider a combination. Party A is a laundry facilities management company.</t>
+          <t>BofA, as instructed by the Board, called Party A (a laundry facilities management company) about a possible combination; Party A said it might consider one. First contact with Party A.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>“representatives of BofA Merrill Lynch, as instructed by the Board, telephoned a representative of Party A to discuss generally a possible business combination between Party A and Mac-Gray.” (p. 27)</t>
+          <t>“the representative of Party A indicated that Party A might consider a business combination with Mac-Gray” (p. 27)</t>
         </is>
       </c>
       <c r="R3" s="2" t="n"/>
@@ -732,12 +733,12 @@
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Target's outside legal counsel, first seen acting here. Later also advised the Special Committee.</t>
+          <t>Mac-Gray's outside legal counsel; first seen acting at the 05/09 Board meeting. Later also advised the Special Committee.</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>“representatives from BofA Merrill Lynch and Goodwin Procter LLP, outside legal counsel to Mac-Gray, were also in attendance” (p. 27)</t>
+          <t>“Goodwin Procter LLP, outside legal counsel to Mac-Gray” (p. 27)</t>
         </is>
       </c>
       <c r="R4" s="2" t="n"/>
@@ -758,18 +759,18 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>05/15/2013</t>
+          <t>05/09/2013</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>BofA Merrill Lynch</t>
+          <t>Mac-Gray</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Adviser ended</t>
+          <t>Target sale decision</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -788,24 +789,24 @@
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>The Transaction Committee decided on 05/14 to end the 2011-2012 mandate, since BofA was being invited to pitch for the sale-review role.</t>
+          <t>Board discussed a possible sale process and its risks (leaks, disclosure to competitors); formed a Transaction Committee (Bullock, Daoust) to recommend a financial adviser for a strategic-alternatives review incl. a sale. Qualification: sale-process decision deferred.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>“Mac-Gray sent a letter to BofA Merrill Lynch terminating their engagement in connection with the 2011-2012 Discussions.” (p. 29)</t>
+          <t>“The Board concluded that it would discuss the review of strategic alternatives, including engaging in a potential sale process, at its next meeting” (p. 28)</t>
         </is>
       </c>
       <c r="R5" s="2" t="n"/>
       <c r="S5" s="2" t="n"/>
       <c r="T5" s="3" t="n">
-        <v>41409</v>
+        <v>41403</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>41409</v>
+        <v>41403</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>41409</v>
+        <v>41403</v>
       </c>
     </row>
     <row r="6">
@@ -814,7 +815,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>05/30/2013</t>
+          <t>05/15/2013</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -825,7 +826,7 @@
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Adviser ended</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -844,24 +845,24 @@
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Re-engaged as the target's sole financial adviser for the strategic review and possible sale, chosen from three banks. Engagement letter 05/31; no buyer financing without consent.</t>
+          <t>Mac-Gray terminated BofA's 2011–2012 Discussions engagement letter (Transaction Committee decision 05/14), because BofA was to pitch for the new sale mandate and the CSC sale had ended.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>“the Board unanimously approved the engagement of BofA Merrill Lynch on the terms discussed at this meeting.” (p. 29)</t>
+          <t>“Mac-Gray sent a letter to BofA Merrill Lynch terminating their engagement in connection with the 2011-2012 Discussions” (p. 29)</t>
         </is>
       </c>
       <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="3" t="n">
-        <v>41424</v>
+        <v>41409</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>41424</v>
+        <v>41409</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>41424</v>
+        <v>41409</v>
       </c>
     </row>
     <row r="7">
@@ -875,13 +876,13 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Moab Partners, L.P.</t>
+          <t>BofA Merrill Lynch</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Activist</t>
+          <t>Adviser</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -900,12 +901,12 @@
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Moab (about 9% holder) won a proxy contest; Rothenberg and Hyman replaced incumbents. The filing does not say Moab pressed for a sale. Rothenberg was later excluded over Moab's rollover interest.</t>
+          <t>Re-engaged as Mac-Gray's (sole) financial adviser for the strategic-alternatives review incl. a sale, chosen over two other banks (pitches 05/22, 05/29). Letter signed 05/31 bars it from financing buyers without consent. Fee about $8.1m (p. 51).</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>“the Mac-Gray stockholders elected as directors Michael M. Rothenberg and James E. Hyman, candidates nominated by Mac-Gray's stockholder, Moab Partners, L.P.” (p. 29)</t>
+          <t>“the Board unanimously approved the engagement of BofA Merrill Lynch on the terms discussed at this meeting” (p. 29)</t>
         </is>
       </c>
       <c r="R7" s="2" t="n"/>
@@ -926,22 +927,18 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>06/21/2013</t>
+          <t>05/30/2013</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Moab Partners, L.P. (Moab)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Activist</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -950,52 +947,34 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Unsolicited proposal to the board, made before any NDA or diligence (Heavy by context). It was still standing when round 1 was evaluated on 07/25.</t>
+          <t>Moab (about 9% holder, per 06/12) won a proxy contest: its nominees Rothenberg (Moab general partner) and Hyman joined the Board. Moab later sought a possible equity rollover (#18, #49); Rothenberg excluded from sale deliberations.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>“Party A submitted an unsolicited proposal to the Mac-Gray Board of Directors offering to purchase Mac-Gray for an all-cash purchase price of $17.00 to $19.00 per share” (p. 30)</t>
+          <t>“the Mac-Gray stockholders elected as directors Michael M. Rothenberg and James E. Hyman, candidates nominated by Mac-Gray's stockholder, Moab Partners, L.P.” (p. 29)</t>
         </is>
       </c>
       <c r="R8" s="2" t="n"/>
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="3" t="n">
-        <v>41446</v>
+        <v>41424</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>41446</v>
+        <v>41424</v>
       </c>
       <c r="V8" s="3" t="n">
-        <v>41446</v>
+        <v>41424</v>
       </c>
     </row>
     <row r="9">
@@ -1004,18 +983,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>06/24/2013</t>
+          <t>06/21/2013</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (Special Committee)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Target sale decision</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1024,34 +1007,56 @@
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
+      <c r="H9" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Board forms a Special Committee of six independent directors, excluding CEO MacDonald and Moab's Rothenberg. The committee will weigh a sale against staying stand-alone and approach 50 parties.</t>
+          <t>Diligence open per narrative: no confidentiality agreement or diligence until 08/05 (#27). Unsolicited written proposal to the Board; Party A enters the process. Financing not stated.</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee concluded that it would be in the best interests of stockholders to consider a potential sale of Mac-Gray” (p. 31)</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="n"/>
+          <t>“Party A submitted an unsolicited proposal to the Mac-Gray Board of Directors offering to purchase Mac-Gray for an all-cash purchase price of $17.00 to $19.00 per share” (p. 30)</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S9" s="2" t="n"/>
       <c r="T9" s="3" t="n">
-        <v>41449</v>
+        <v>41446</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>41449</v>
+        <v>41446</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>41449</v>
+        <v>41446</v>
       </c>
     </row>
     <row r="10">
@@ -1060,25 +1065,25 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>06/24/2013 to 06/28/2013</t>
+          <t>06/24/2013</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (BofA Merrill Lynch)</t>
+          <t>Mac-Gray</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Target sale decision</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -1090,28 +1095,24 @@
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>BofA's outreach carries out the 06/24 decision; contacts reported by 06/28. NDA signers get an informational package, with preliminary IOIs due 07/23/2013 (no separate Deadline set row).</t>
+          <t>Board excluded CEO MacDonald and Rothenberg (possible rollover partners) and formed a six-member independent Special Committee. Committee decided to consider a sale against the stand-alone plan and to approach 50 parties (15 strategic, 35 financial). Projections presented.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>“BofA Merrill Lynch contacted the strategic and financial parties identified at the June 24th Special Committee meeting” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+          <t>“the Special Committee concluded that it would be in the best interests of stockholders to consider a potential sale of Mac-Gray” (p. 31)</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="n"/>
       <c r="S10" s="2" t="n"/>
       <c r="T10" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="U10" s="3" t="n">
         <v>41449</v>
       </c>
       <c r="V10" s="3" t="n">
-        <v>41453</v>
+        <v>41449</v>
       </c>
     </row>
     <row r="11">
@@ -1120,22 +1121,18 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>by 06/28/2013</t>
+          <t>06/24/2013–06/28/2013 (outreach begins)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -1149,25 +1146,27 @@
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated. Pamplona is interested, including an acquisition by its portfolio company CSC (acquired May 2013), and says diligence would be minimal.</t>
+          <t>BofA began contacting the 50 parties chosen on 06/24 over the following weeks; calls with Party A and Pamplona reported by 06/28. Confidentiality signers received an information package and a request for preliminary indications (#16).</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>“BofA Merrill Lynch also reported that they had spoken with representatives of Pamplona, as instructed by the Special Committee, who expressed interest in a transaction” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R11" s="2" t="n"/>
+          <t>“BofA Merrill Lynch contacted the strategic and financial parties identified at the June 24th Special Committee meeting” (p. 32)</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="U11" s="3" t="n">
         <v>41449</v>
@@ -1182,7 +1181,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>during the next several weeks after 06/24/2013</t>
+          <t>during the several weeks after 06/24/2013</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1218,18 +1217,18 @@
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Target outreach. Of 50 contacted (15 strategic, 35 financial), Party A (#2) and CSC/Pamplona (#10) are recorded separately, leaving 13 strategic parties.</t>
+          <t>Target outreach. Total 50 = 15 strategic + 35 financial, incl. Party A (first contacted 04/08, #2; spoke again 06/28, citing synergies and financing sources) and CSC/Pamplona (#14): 15 − 2 = 13. Responses not reported.</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>“to solicit potential interest in a transaction with Mac-Gray, 15 of which were potential strategic buyers and 35 of which were potential financial buyers” (p. 32)</t>
+          <t>“50 parties, including CSC and Pamplona, who together we refer to as CSC/Pamplona, and Party A, to solicit potential interest in a transaction with Mac-Gray” (p. 32)</t>
         </is>
       </c>
       <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
       <c r="T12" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="U12" s="3" t="n">
         <v>41449</v>
@@ -1242,12 +1241,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>during the next several weeks after 06/24/2013</t>
+          <t>during the several weeks after 06/24/2013</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>35 financial parties</t>
+          <t>35 financial parties (incl. Party B, Party C)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1278,18 +1277,22 @@
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Target outreach to all 35 financial parties (including private equity), among them Party B and Party C. 50 contacted in total.</t>
+          <t>Target outreach to 35 financial buyers, incl. private equity firms. Party B and Party C assumed to be among them (filing does not say so expressly; Q4). Rows reconcile to 50: 35 + 13 (#11) + CSC/Pamplona + Party A.</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>“to solicit potential interest in a transaction with Mac-Gray, 15 of which were potential strategic buyers and 35 of which were potential financial buyers” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R13" s="2" t="n"/>
+          <t>“15 of which were potential strategic buyers and 35 of which were potential financial buyers, including private equity firms” (p. 32)</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="n"/>
       <c r="T13" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="U13" s="3" t="n">
         <v>41449</v>
@@ -1302,7 +1305,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>over the two months after late June 2013</t>
+          <t>06/24/2013–08/24/2013 (over the next two months)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1338,7 +1341,7 @@
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>20 NDAs in total (2 strategic, 18 financial). Party A, CSC/Pamplona, Party B and Party C have their own rows, leaving 16 financial. Signing dates not given; each got an informational package.</t>
+          <t>Filing total: 20 signers over two months = 2 strategic (Party A #27, CSC/Pamplona #19) + 18 financial incl. Party B (#15), Party C (#17); residual 18 − 2 = 16. Dates not reported. Standstills had sunset provisions. Each received the information package.</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -1348,17 +1351,19 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
       <c r="T14" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="U14" s="3" t="n">
         <v>41449</v>
       </c>
-      <c r="V14" s="2" t="n"/>
+      <c r="V14" s="3" t="n">
+        <v>41510</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1366,22 +1371,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>06/28/2013</t>
+          <t>by 06/28/2013</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1402,21 +1407,21 @@
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Confidentiality and standstill agreement; received the informational package.</t>
+          <t>BofA, as instructed, called Pamplona, which was interested incl. in an acquisition by its portfolio company CSC; said diligence would be minimal given its familiarity. One bidder unit; filing classes it strategic.</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>“Party B, entered into a confidentiality and standstill agreement with Mac-Gray” (p. 32)</t>
+          <t>“Pamplona emphasized that business and legal due diligence would be minimal given its familiarity with Mac-Gray and the industry generally” (p. 32)</t>
         </is>
       </c>
       <c r="R15" s="2" t="n"/>
       <c r="S15" s="2" t="n"/>
       <c r="T15" s="3" t="n">
-        <v>41453</v>
+        <v>41451</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>41453</v>
+        <v>41449</v>
       </c>
       <c r="V15" s="3" t="n">
         <v>41453</v>
@@ -1428,12 +1433,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>06/30/2013</t>
+          <t>06/28/2013</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>Party B</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1464,24 +1469,24 @@
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Confidentiality and standstill agreement; received the informational package.</t>
+          <t>Enters: confidentiality and standstill agreement; received the information package for a preliminary indication. Financial bidder (p. 32).</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>“Party C entered into a confidentiality and standstill agreement with Mac-Gray” (p. 32)</t>
+          <t>“Party B, entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 32)</t>
         </is>
       </c>
       <c r="R16" s="2" t="n"/>
       <c r="S16" s="2" t="n"/>
       <c r="T16" s="3" t="n">
-        <v>41455</v>
+        <v>41453</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>41455</v>
+        <v>41453</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>41455</v>
+        <v>41453</v>
       </c>
     </row>
     <row r="17">
@@ -1490,18 +1495,18 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>07/06/2013</t>
+          <t>06/28/2013 (with information packages)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (Special Committee)</t>
+          <t>Mac-Gray</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Deadline set</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -1517,27 +1522,35 @@
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Refuses rollover partnership: denies the request (relayed by Rothenberg 07/03) for Moab to partner exclusively with CSC/Pamplona on a rollover. Such talks allowed only later.</t>
+          <t>Preliminary indications due 07/23/2013, to address valuation, financing, conditions and diligence focus. The instruction came with each signer's information package; dated at the first reported package (Party B, #15).</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee decided to deny the exclusivity request at this stage of the process” (p. 33)</t>
-        </is>
-      </c>
-      <c r="R17" s="2" t="n"/>
+          <t>“which they were instructed to submit by July 23, 2013” (p. 32)</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="n"/>
       <c r="T17" s="3" t="n">
-        <v>41461</v>
+        <v>41453</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>41461</v>
+        <v>41453</v>
       </c>
       <c r="V17" s="3" t="n">
-        <v>41461</v>
+        <v>41453</v>
       </c>
     </row>
     <row r="18">
@@ -1546,17 +1559,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>07/11/2013</t>
+          <t>06/30/2013</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
+          <t>Party C</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1582,24 +1595,24 @@
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Agreement with Pamplona Capital Management LLC, reused in the merger agreement (s. 6.17). Received the informational package. Party A's NDA talks stalled on non-solicit terms 07/11-07/23.</t>
+          <t>Enters: confidentiality and standstill agreement; received the information package. Financial bidder (p. 32).</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona entered into a confidentiality and standstill agreement with Mac-Gray” (p. 33)</t>
+          <t>“Party C entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 32)</t>
         </is>
       </c>
       <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="3" t="n">
-        <v>41466</v>
+        <v>41455</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>41466</v>
+        <v>41455</v>
       </c>
       <c r="V18" s="3" t="n">
-        <v>41466</v>
+        <v>41455</v>
       </c>
     </row>
     <row r="19">
@@ -1608,22 +1621,18 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>07/23/2013</t>
+          <t>07/06/2013</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -1632,52 +1641,34 @@
       <c r="G19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="4" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Preliminary IOI based only on the informational package, with no data room or management access (Heavy by context).</t>
+          <t>Refused rollover partnership: on 07/03 Rothenberg said Pamplona would seek confidentiality terms letting CSC/Pamplona share its bid and data with Moab, Moab dealing exclusively with them. Special Committee refused; rollover talks premature with anyone, allowed later.</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a preliminary indication of interest at an all-cash purchase price of $18.50 per share.” (p. 33)</t>
+          <t>“the Special Committee decided to deny the exclusivity request at this stage of the process” (p. 33)</t>
         </is>
       </c>
       <c r="R19" s="2" t="n"/>
       <c r="S19" s="2" t="n"/>
       <c r="T19" s="3" t="n">
-        <v>41478</v>
+        <v>41461</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>41478</v>
+        <v>41461</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>41478</v>
+        <v>41461</v>
       </c>
     </row>
     <row r="20">
@@ -1686,18 +1677,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>07/23/2013</t>
+          <t>07/11/2013</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n"/>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -1711,33 +1706,31 @@
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
+      <c r="M20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Due date for preliminary IOIs. CSC/Pamplona bid on time; Party B and Party C bid on 07/24 and were considered on 07/25 (late bids accepted).</t>
+          <t>Enters: confidentiality and standstill agreement signed by CSC/Pamplona; received the information package. CSC is a laundry operator owned by Pamplona (private equity fund).</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>“a preliminary indication of interest, which they were instructed to submit by July 23, 2013” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+          <t>“CSC/Pamplona entered into a confidentiality and standstill agreement with Mac-Gray and were provided with an informational package” (p. 33)</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
       <c r="T20" s="3" t="n">
-        <v>41478</v>
+        <v>41466</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>41478</v>
+        <v>41466</v>
       </c>
       <c r="V20" s="3" t="n">
-        <v>41478</v>
+        <v>41466</v>
       </c>
     </row>
     <row r="21">
@@ -1751,17 +1744,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>16 other financial NDA signers</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Did not submit</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -1770,39 +1763,43 @@
       <c r="G21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
+      <c r="H21" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Inferred. 20 signers − Party A (no NDA until 08/05) − 3 submitters = 16. On 07/25 the target named only four interested bidders. Some may have signed after 07/23.</t>
+          <t>Diligence open per narrative: management presentation 08/12; limited data-room access, customer data reserved (#28). Preliminary indication; financing and conditions not stated.</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>“reach out to each of the four interested bidders and arrange management meetings” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
+          <t>“CSC/Pamplona submitted a preliminary indication of interest at an all-cash purchase price of $18.50 per share” (p. 33)</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="n"/>
       <c r="S21" s="2" t="n"/>
       <c r="T21" s="3" t="n">
         <v>41478</v>
@@ -1820,22 +1817,18 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>07/24/2013</t>
+          <t>07/23/2013</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -1844,52 +1837,38 @@
       <c r="G22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Written preliminary IOI, one day after the due date. Based on the informational package only (Heavy by context).</t>
+          <t>Preliminary indications due. CSC/Pamplona on time (#20); late: Party B and Party C on 07/24 (#22, #23), Party C written revision 07/25 (#26); all reviewed 07/25. No bids reported from the other 16 signers.</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>“Party B submitted a preliminary indication of interest at an all-cash purchase price of $17.00 to $18.00 per share.” (p. 33)</t>
-        </is>
-      </c>
-      <c r="R22" s="2" t="n"/>
+          <t>“which they were instructed to submit by July 23, 2013” (p. 32)</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="n"/>
       <c r="T22" s="3" t="n">
-        <v>41479</v>
+        <v>41478</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>41479</v>
+        <v>41478</v>
       </c>
       <c r="V22" s="3" t="n">
-        <v>41479</v>
+        <v>41478</v>
       </c>
     </row>
     <row r="23">
@@ -1903,7 +1882,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>Party B</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1923,10 +1902,10 @@
         <v>1</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -1940,7 +1919,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Heavy</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="M23" s="2" t="n">
@@ -1950,15 +1929,19 @@
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Oral preliminary IOI to BofA, one day after the due date. Based on the informational package only (Heavy by context).</t>
+          <t>Diligence open per narrative: management presentation 08/06; data-room diligence 08/06–08/27. Preliminary indication, one day after the 07/23 due date. Financing not stated.</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>“presented an oral preliminary indication of interest at an all-cash purchase price of $15.00 to $17.00 per share” (p. 33)</t>
-        </is>
-      </c>
-      <c r="R23" s="2" t="n"/>
+          <t>“Party B submitted a preliminary indication of interest at an all-cash purchase price of $17.00 to $18.00 per share” (p. 33)</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S23" s="2" t="n"/>
       <c r="T23" s="3" t="n">
         <v>41479</v>
@@ -1976,58 +1959,80 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>07/25/2013</t>
+          <t>07/24/2013</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (Special Committee)</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="n"/>
+          <t>Party C</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Committee finds IOIs lower than expected. Advances four: Party A (subject to NDA), Party B, Party C, CSC/Pamplona. Staged disclosure; management meetings for all, synergy information for strategics; revised IOIs to follow.</t>
+          <t>Diligence open per narrative: management presentation 08/08. Oral preliminary indication by phone to BofA, one day after the due date.</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>“authorized and instructed BofA Merrill Lynch to proceed with the staged disclosure as discussed at this meeting and to reach out to each of the four interested bidders” (p. 34)</t>
+          <t>“representatives from Party C called BofA Merrill Lynch and presented an oral preliminary indication of interest at an all-cash purchase price of $15.00 to $17.00 per share” (p. 33)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S24" s="2" t="n"/>
       <c r="T24" s="3" t="n">
-        <v>41480</v>
+        <v>41479</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>41480</v>
+        <v>41479</v>
       </c>
       <c r="V24" s="3" t="n">
-        <v>41480</v>
+        <v>41479</v>
       </c>
     </row>
     <row r="25">
@@ -2036,12 +2041,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>07/25/2013</t>
+          <t>by 07/25/2013</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>16 other financial NDA signers</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2051,7 +2056,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -2060,50 +2065,44 @@
       <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="I25" s="4" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Written IOI after the 07/25 meeting; revises #22 (oral $15.00-$17.00). Answers the round-1 request. Based on the informational package only (Heavy by context).</t>
+          <t>Not among the four bidders advanced on 07/25 (#25); no bids from them reported. 20 signers − 4 advanced = 16. Signing dates unknown: any later signer was outside the four-bidder stage (08/27 letters to four only). Q4.</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>“Party C submitted a written indication of interest at an all-cash purchase price of $16.00 to $16.50 per share.” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R25" s="2" t="n"/>
+          <t>“reach out to each of the four interested bidders and arrange management meetings” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
       <c r="S25" s="2" t="n"/>
       <c r="T25" s="3" t="n">
         <v>41480</v>
       </c>
-      <c r="U25" s="3" t="n">
-        <v>41480</v>
-      </c>
+      <c r="U25" s="2" t="n"/>
       <c r="V25" s="3" t="n">
         <v>41480</v>
       </c>
@@ -2114,22 +2113,18 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>08/05/2013</t>
+          <t>07/25/2013</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -2143,31 +2138,33 @@
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Talks resumed 07/27 and non-solicit terms agreed. Received the informational package so it could improve its 06/21 proposal (#7).</t>
+          <t>Committee found indications low; chose staged disclosure and advanced four: Party A (if it signed a confidentiality agreement), Party B, Party C, CSC/Pamplona, for management meetings (held 08/06–08/14 for all four), then revised indications.</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>“Party A entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R26" s="2" t="n"/>
+          <t>“authorized and instructed BofA Merrill Lynch to proceed with the staged disclosure as discussed at this meeting and to reach out to each of the four interested bidders” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="3" t="n">
-        <v>41491</v>
+        <v>41480</v>
       </c>
       <c r="U26" s="3" t="n">
-        <v>41491</v>
+        <v>41480</v>
       </c>
       <c r="V26" s="3" t="n">
-        <v>41491</v>
+        <v>41480</v>
       </c>
     </row>
     <row r="27">
@@ -2176,54 +2173,80 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>08/06/2013 to 08/27/2013</t>
+          <t>07/25/2013</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n"/>
+          <t>Party C</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Information access differs by bidder type: B and C (financial) get broad data-room access; A and CSC/Pamplona (strategic) get limited access, customer data withheld, plus synergy talks. All four had management presentations 08/06-08/14.</t>
+          <t>Diligence open per narrative: management presentation 08/08. Written indication after the committee meeting, replacing the oral range (#23): top cut from $17.00 to $16.50.</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>“Party A and CSC/Pamplona, in light of the fact that they were strategic bidders, were given somewhat limited access to this electronic data site” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R27" s="2" t="n"/>
+          <t>“Party C submitted a written indication of interest at an all-cash purchase price of $16.00 to $16.50 per share” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S27" s="2" t="n"/>
       <c r="T27" s="3" t="n">
-        <v>41492</v>
+        <v>41480</v>
       </c>
       <c r="U27" s="3" t="n">
-        <v>41492</v>
+        <v>41480</v>
       </c>
       <c r="V27" s="3" t="n">
-        <v>41513</v>
+        <v>41480</v>
       </c>
     </row>
     <row r="28">
@@ -2232,18 +2255,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>08/27/2013</t>
+          <t>08/05/2013</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (BofA Merrill Lynch)</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Deadline set</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -2257,29 +2284,35 @@
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="n"/>
+      <c r="M28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Letter to all four (authorized 08/15): revised written proposals due 09/09/2013 to go on to in-depth evaluation. Proposals to cover valuation, financing, approvals, covenants and diligence.</t>
+          <t>Catch-up access: after talks on non-solicitation terms stalled (07/11–07/23) and resumed 07/27 (filing prints '2103'), Party A signed and got the information package to improve its 06/21 proposal (#8). Already entered at #8.</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>“instructing such bidders to submit revised written proposals no later than September 9, 2013 if such bidders wished to proceed further in the process” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R28" s="2" t="n"/>
+          <t>“Party A entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="3" t="n">
-        <v>41513</v>
+        <v>41491</v>
       </c>
       <c r="U28" s="3" t="n">
-        <v>41513</v>
+        <v>41491</v>
       </c>
       <c r="V28" s="3" t="n">
-        <v>41513</v>
+        <v>41491</v>
       </c>
     </row>
     <row r="29">
@@ -2288,22 +2321,18 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>09/09/2013</t>
+          <t>between 08/06/2013 and 08/27/2013</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -2312,52 +2341,38 @@
       <c r="G29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="4" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Revised IOI, up from $18.50 (#18). Pamplona commits 100% of the capital. Requests 2-week exclusivity. Heavy: customer data still withheld and further in-depth diligence expected.</t>
+          <t>Staged information access: financial bidders Party B and Party C got broad data-room access; strategic bidders Party A and CSC/Pamplona got limited access, customer data incl. locations reserved for later (07/25 staging). Strategics also discussed synergies with management.</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a revised indication of interest with an all-cash purchase price of $19.50 per share, indicating that Pamplona was committed to provide 100% of the capital” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R29" s="2" t="n"/>
+          <t>“Party B and Party C, in light of the fact that they were financial bidders, were given broad access to an electronic data site” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="3" t="n">
-        <v>41526</v>
+        <v>41492</v>
       </c>
       <c r="U29" s="3" t="n">
-        <v>41526</v>
+        <v>41492</v>
       </c>
       <c r="V29" s="3" t="n">
-        <v>41526</v>
+        <v>41513</v>
       </c>
     </row>
     <row r="30">
@@ -2366,22 +2381,18 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>09/09/2013</t>
+          <t>08/27/2013</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline set</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -2390,52 +2401,38 @@
       <c r="G30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H30" s="4" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="I30" s="4" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Revised IOI, up from $17.00-$18.00 (#21). Financing from affiliated-fund equity plus third-party debt; no firm financing commitment (Heavy).</t>
+          <t>BofA letters to Party A, Party B, Party C and CSC/Pamplona (authorized 08/15): revised written proposals due 09/09/2013 to go on to in-depth evaluation; address valuation, financing, approvals, covenants, diligence focus.</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>“Party B also submitted a revised indication of interest with an all-cash purchase price of $18.50 per share” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R30" s="2" t="n"/>
+          <t>“instructing such bidders to submit revised written proposals no later than September 9, 2013 if such bidders wished to proceed further in the process” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="3" t="n">
-        <v>41526</v>
+        <v>41513</v>
       </c>
       <c r="U30" s="3" t="n">
-        <v>41526</v>
+        <v>41513</v>
       </c>
       <c r="V30" s="3" t="n">
-        <v>41526</v>
+        <v>41513</v>
       </c>
     </row>
     <row r="31">
@@ -2449,13 +2446,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="n"/>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -2464,29 +2465,43 @@
       <c r="G31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
+      <c r="H31" s="4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Due date for revised written proposals. CSC/Pamplona and Party B bid on time; Party A and Party C bid on 09/10 and were reviewed on 09/11 (late bids accepted).</t>
+          <t>Diligence open per narrative: customer data still reserved; diligence continued 09/11–09/18. Pamplona committed to provide 100% of capital. Requested two-week exclusivity. Revised indication.</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>“instructing such bidders to submit revised written proposals no later than September 9, 2013” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+          <t>“CSC/Pamplona submitted a revised indication of interest with an all-cash purchase price of $19.50 per share, indicating that Pamplona was committed to provide 100% of the capital” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="n"/>
       <c r="S31" s="2" t="n"/>
       <c r="T31" s="3" t="n">
         <v>41526</v>
@@ -2504,17 +2519,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>09/10/2013</t>
+          <t>09/09/2013</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
+          <t>Party B</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2529,10 +2544,10 @@
         <v>2</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
@@ -2556,24 +2571,24 @@
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Revised IOI, one day late; same range as its 06/21 proposal (#7). To be financed by existing credit facilities or affiliated equity; no firm financing commitment (Heavy).</t>
+          <t>No firm financing commitment: to be financed by affiliated-fund equity plus third-party debt (p. 35). Revised indication.</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>“Party A submitted a revised indication of interest with an all-cash purchase price of $18.00 to $19.00 per share, to be financed by outstanding credit facilities or affiliated equity sources.” (p. 35)</t>
+          <t>“Party B also submitted a revised indication of interest with an all-cash purchase price of $18.50 per share” (p. 35)</t>
         </is>
       </c>
       <c r="R32" s="2" t="n"/>
       <c r="S32" s="2" t="n"/>
       <c r="T32" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
       <c r="U32" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
       <c r="V32" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
     </row>
     <row r="33">
@@ -2582,22 +2597,18 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>09/10/2013</t>
+          <t>09/09/2013</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -2606,52 +2617,38 @@
       <c r="G33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H33" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>Revised oral IOI to BofA, one day late; revises #24 ($16.00-$16.50). No firm financing commitment (Heavy).</t>
+          <t>Revised proposals due. CSC/Pamplona and Party B on time (#30, #31); late: Party A and Party C on 09/10 (#33, #34), all reviewed by the committee 09/11.</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>“indicated that it was submitting a revised oral indication of interest with an all-cash purchase price of $16.00 to $17.00 per share” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R33" s="2" t="n"/>
+          <t>“submit revised written proposals no later than September 9, 2013” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="n"/>
       <c r="T33" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
       <c r="U33" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
       <c r="V33" s="3" t="n">
-        <v>41527</v>
+        <v>41526</v>
       </c>
     </row>
     <row r="34">
@@ -2660,18 +2657,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>09/11/2013</t>
+          <t>09/10/2013</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Stewart G. MacDonald, Jr. (CEO)</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -2680,34 +2681,56 @@
       <c r="G34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
+      <c r="H34" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Rollover refused by holder: CEO and major holder says he won't roll over shares. BofA reports bidders unlikely to proceed without his support; committee has him fully briefed (09/12). He backs the process, wants higher value.</t>
+          <t>No firm financing commitment (p. 35); to be funded by existing credit facilities or affiliated equity. Revised indication, one day late; floor raised from $17.00 (#8).</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>“it was unlikely that any of these parties would move forward in the process without the express support of Mr. MacDonald” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="n"/>
+          <t>“Party A submitted a revised indication of interest with an all-cash purchase price of $18.00 to $19.00 per share, to be financed by outstanding credit facilities or affiliated equity sources” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S34" s="2" t="n"/>
       <c r="T34" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
       <c r="U34" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
       <c r="V34" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
     </row>
     <row r="35">
@@ -2716,58 +2739,80 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>09/11/2013</t>
+          <t>09/10/2013</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (Special Committee)</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="n"/>
+          <t>Party C</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
-      <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>BofA calls all four the same day asking for final IOIs by 09/18/2013. Short exclusivity offered to one bidder depending on price and deal certainty.</t>
+          <t>No firm financing commitment (p. 35). Oral revised indication by phone to BofA, one day late; up from $16.00–16.50 (#26).</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee instructed BofA Merrill Lynch to call each of Party A, Party B, Party C and CSC/Pamplona to request final indications of interest by September 18, 2013” (p. 36)</t>
+          <t>“a representative of Party C indicated that it was submitting a revised oral indication of interest with an all-cash purchase price of $16.00 to $17.00 per share” (p. 35)</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
       <c r="U35" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
       <c r="V35" s="3" t="n">
-        <v>41528</v>
+        <v>41527</v>
       </c>
     </row>
     <row r="36">
@@ -2776,80 +2821,54 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>09/18/2013</t>
+          <t>09/11/2013</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Stewart G. MacDonald, Jr. (CEO, large holder)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>20.75</v>
-      </c>
-      <c r="I36" s="4" t="n">
-        <v>20.75</v>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>Formal</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Final-round proposal, up from $19.50 (#28); Formal as a response to the final solicitation. Pamplona commits 100% of the capital; only confirmatory diligence followed (Light). Requests 2-week exclusivity.</t>
+          <t>Rollover refused by holder: MacDonald said he would not roll over shares. BofA reported bidders unlikely to proceed without his express support, so the committee had him fully briefed (09/12); he backed continuing but urged a higher value.</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a proposal for an all-cash purchase price of $20.75 per share, reiterating that Pamplona was committed to provide 100% of the capital” (p. 36)</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
+          <t>“Mr. MacDonald indicated that he had decided that he was not interested in rolling over any of his shares in any transaction” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="n"/>
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
       <c r="U36" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
       <c r="V36" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
     </row>
     <row r="37">
@@ -2858,22 +2877,18 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>09/18/2013</t>
+          <t>09/11/2013</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Bid reaffirmed</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -2882,56 +2897,38 @@
       <c r="G37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="I37" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>Formal</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>Heavy</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>By phone to BofA: confirms #31 as its best and final offer, answering the final solicitation. The 09/10 bid had no firm financing commitment and none is reported since (Heavy).</t>
+          <t>Committee had BofA call all four (Party A, Party B, Party C, CSC/Pamplona) the same day for final indications due 09/18/2013, saying Mac-Gray might grant one bidder short exclusivity depending on price and deal certainty.</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>“its previous indication of interest with an all-cash purchase price of $18.00 to $19.00 per share was its best and final offer” (p. 36)</t>
+          <t>“request final indications of interest by September 18, 2013” (p. 36)</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S37" s="2" t="n"/>
       <c r="T37" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
       <c r="U37" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
       <c r="V37" s="3" t="n">
-        <v>41535</v>
+        <v>41528</v>
       </c>
     </row>
     <row r="38">
@@ -2945,12 +2942,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2965,14 +2962,14 @@
         <v>3</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>21.5</v>
+        <v>20.75</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>21.5</v>
+        <v>20.75</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2982,7 +2979,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Heavy</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="M38" s="2" t="n">
@@ -2992,17 +2989,17 @@
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Party B values its bid at $21.50: $19.00 cash plus options for 10% of new equity, which it values at $2.50 and which vest on a five-year target. Debt-and-equity financing, no commitment reported (Heavy).</t>
+          <t>Diligence open per narrative: customer data still reserved (#28, #48). Pamplona committed to provide 100% of capital; requested two-week exclusivity. Formal as the answer to the final-indication request, no markup (Q3).</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>“Party B also submitted a revised indication of interest with a purchase price that Party B valued at $21.50 per share, including $19.00 of cash to be paid at closing” (p. 36)</t>
+          <t>“CSC/Pamplona submitted a proposal for an all-cash purchase price of $20.75 per share, reiterating that Pamplona was committed to provide 100% of the capital” (p. 36)</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Q4; Q5</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="S38" s="2" t="n"/>
@@ -3027,17 +3024,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>Party A</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Did not submit</t>
+          <t>Bid reaffirmed</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -3046,31 +3043,47 @@
       <c r="G39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
+      <c r="H39" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
+      <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Did not submit or reaffirm its $16.00-$17.00 IOI (#32) and gave no reason. Reported on 09/19; not seen again.</t>
+          <t>Diligence open per narrative: customer data reserved; diligence continued 09/11–09/18. By price confirmation: Party A told BofA by phone its 09/10 range (#33) was its best and final offer. Financing status at this date not reported.</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>“Party C did not submit a revised indication of interest or reiterate its prior indication of interest” (p. 36)</t>
-        </is>
-      </c>
-      <c r="R39" s="2" t="n"/>
+          <t>“its previous indication of interest with an all-cash purchase price of $18.00 to $19.00 per share was its best and final offer” (p. 36)</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
       <c r="S39" s="2" t="n"/>
       <c r="T39" s="3" t="n">
         <v>41535</v>
@@ -3093,13 +3106,17 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="n"/>
+          <t>Party B</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -3108,27 +3125,45 @@
       <c r="G40" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
+      <c r="H40" s="4" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Due date for final IOIs, reached. On 09/19 the committee acted on the bids in hand (enforced).</t>
+          <t>Diligence open per narrative: diligence continued 09/11–09/18. Bidder values offer at $21.50: $19.00 cash at closing plus options on 10% of new equity, vesting on base-case projections over five years, valued by it at $2.50. Committee expected affiliated equity plus third-party debt (p. 37). Q5.</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>“request final indications of interest by September 18, 2013” (p. 36)</t>
+          <t>“a revised indication of interest with a purchase price that Party B valued at $21.50 per share, including $19.00 of cash to be paid at closing” (p. 36)</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3; Q5</t>
         </is>
       </c>
       <c r="S40" s="2" t="n"/>
@@ -3148,18 +3183,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>09/19/2013</t>
+          <t>09/18/2013</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray (Special Committee)</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="n"/>
+          <t>Party C</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Did not submit</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -3173,29 +3212,35 @@
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
-      <c r="M41" s="2" t="n"/>
-      <c r="N41" s="2" t="n"/>
+      <c r="M41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Preferred bidder and price requirement: CSC/Pamplona is best on value, certainty and risk (Party B's options and financing riskier). Exclusivity offered at $21.25; MacDonald supports $21.25.</t>
+          <t>Party C neither revised nor reiterated its $16.00–17.00 indication (#34) by the final-indication due date and gave no reason. Its decision.</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee would be prepared to move into exclusivity at a price of $21.25 per share” (p. 37)</t>
+          <t>“Party C did not submit a revised indication of interest or reiterate its prior indication of interest” (p. 36)</t>
         </is>
       </c>
       <c r="R41" s="2" t="n"/>
       <c r="S41" s="2" t="n"/>
       <c r="T41" s="3" t="n">
-        <v>41536</v>
+        <v>41535</v>
       </c>
       <c r="U41" s="3" t="n">
-        <v>41536</v>
+        <v>41535</v>
       </c>
       <c r="V41" s="3" t="n">
-        <v>41536</v>
+        <v>41535</v>
       </c>
     </row>
     <row r="42">
@@ -3204,22 +3249,18 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>09/21/2013</t>
+          <t>09/18/2013</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -3228,56 +3269,38 @@
       <c r="G42" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="4" t="n">
-        <v>21.25</v>
-      </c>
-      <c r="I42" s="4" t="n">
-        <v>21.25</v>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>Formal</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
+      <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>Raised from $20.75 (#35) the same day the committee asked. Conditioned on 2-week exclusivity; asks for voting agreements from MacDonald. Pamplona funds 100%, no financing contingency; confirmatory diligence only (Light).</t>
+          <t>Final indications due. CSC/Pamplona, Party B and Party A (reaffirmation) answered the same day; Party C did not (#40). Committee chose on the bids in hand on 09/19 (#42).</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona were willing to increase their all-cash purchase price to $21.25 per share as a last and best offer” (p. 37)</t>
+          <t>“request final indications of interest by September 18, 2013” (p. 36)</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S42" s="2" t="n"/>
       <c r="T42" s="3" t="n">
-        <v>41538</v>
+        <v>41535</v>
       </c>
       <c r="U42" s="3" t="n">
-        <v>41538</v>
+        <v>41535</v>
       </c>
       <c r="V42" s="3" t="n">
-        <v>41538</v>
+        <v>41535</v>
       </c>
     </row>
     <row r="43">
@@ -3286,22 +3309,18 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>09/24/2013</t>
+          <t>09/19/2013</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Exclusivity changed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -3315,31 +3334,29 @@
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Executed, authorized 09/23; exclusive until 5 p.m. 10/12/2013. Ends if CSC/Pamplona adversely changes the $21.25 final proposal. CSC/Pamplona then got full data-room access.</t>
+          <t>Preferred bidder and price requirement: committee judged CSC/Pamplona best on value, certainty and no third-party financing, despite Party B's higher face value (option risk); offered exclusivity at $21.25. MacDonald said he would support $21.25.</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013” (p. 38)</t>
+          <t>“the Special Committee would be prepared to move into exclusivity at a price of $21.25 per share” (p. 37)</t>
         </is>
       </c>
       <c r="R43" s="2" t="n"/>
       <c r="S43" s="2" t="n"/>
       <c r="T43" s="3" t="n">
-        <v>41541</v>
+        <v>41536</v>
       </c>
       <c r="U43" s="3" t="n">
-        <v>41541</v>
+        <v>41536</v>
       </c>
       <c r="V43" s="3" t="n">
-        <v>41541</v>
+        <v>41536</v>
       </c>
     </row>
     <row r="44">
@@ -3348,12 +3365,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>by 09/24/2013</t>
+          <t>09/21/2013</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -3363,7 +3380,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -3372,44 +3389,56 @@
       <c r="G44" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
+      <c r="H44" s="4" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>Would not improve earlier offer</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N44" s="2" t="n"/>
+      <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Inferred: displaced when exclusivity with CSC/Pamplona was executed; not reported told. On 09/18 it declined to improve its $18.00-$19.00 range (#36).</t>
+          <t>Diligence open per narrative: customer data not yet released (#48). Pamplona funding 100%, no financing contingency (terms of 09/21–09/23). 'Last and best' answer to #42, conditional on two-week exclusivity; requested MacDonald voting agreements.</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013” (p. 38)</t>
-        </is>
-      </c>
-      <c r="R44" s="2" t="n"/>
+          <t>“willing to increase their all-cash purchase price to $21.25 per share as a last and best offer, provided that Mac-Gray agree to a two week period of exclusive negotiations” (p. 37)</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="3" t="n">
-        <v>41541</v>
+        <v>41538</v>
       </c>
       <c r="U44" s="3" t="n">
-        <v>41541</v>
+        <v>41538</v>
       </c>
       <c r="V44" s="3" t="n">
-        <v>41541</v>
+        <v>41538</v>
       </c>
     </row>
     <row r="45">
@@ -3418,22 +3447,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>by 09/24/2013</t>
+          <t>09/24/2013</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Exclusivity changed</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -3450,24 +3479,16 @@
       <c r="M45" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>Terms or process</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N45" s="2" t="n"/>
+      <c r="O45" s="2" t="n"/>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Inferred date: displaced by exclusivity with CSC/Pamplona. Reason from the committee on 09/19: Party B's options were contingent and deferred, and its financing riskier, despite the higher face value.</t>
+          <t>Executed with CSC and Pamplona to 5 p.m. ET 10/12/2013 (authorized 09/23); lapses if they worsen the final proposal: $21.25 cash, $15m reverse termination fee, no financing contingency, Pamplona funding 100%.</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>“the revised indication of interest submitted by CSC/Pamplona had the potential of delivering the most value to stockholders, provided greater certainty and involved less potential risk” (p. 37)</t>
+          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013” (p. 38)</t>
         </is>
       </c>
       <c r="R45" s="2" t="n"/>
@@ -3488,18 +3509,22 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>09/25/2013</t>
+          <t>by 09/24/2013</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Kirkland &amp; Ellis LLP</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -3513,29 +3538,39 @@
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="n"/>
-      <c r="N46" s="2" t="n"/>
-      <c r="O46" s="2" t="n"/>
+      <c r="M46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Outside legal counsel to CSC/Pamplona; first seen acting when it received the target's first merger agreement draft.</t>
+          <t>Inferred: live rival when exclusivity with CSC/Pamplona was executed (#44); filing does not say it was told. Its best and final $18.00–19.00 (#38) was below CSC/Pamplona's $21.25.</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>“Kirkland &amp; Ellis LLP, outside legal counsel to CSC/Pamplona” (p. 38)</t>
+          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations” (p. 38)</t>
         </is>
       </c>
       <c r="R46" s="2" t="n"/>
       <c r="S46" s="2" t="n"/>
       <c r="T46" s="3" t="n">
-        <v>41542</v>
+        <v>41541</v>
       </c>
       <c r="U46" s="3" t="n">
-        <v>41542</v>
+        <v>41535</v>
       </c>
       <c r="V46" s="3" t="n">
-        <v>41542</v>
+        <v>41541</v>
       </c>
     </row>
     <row r="47">
@@ -3544,18 +3579,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>09/25/2013 to 10/07/2013</t>
+          <t>by 09/24/2013</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Moab Partners, L.P.</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="n"/>
+          <t>Party B</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -3569,29 +3608,39 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
+      <c r="M47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>Rollover resolved: talks with Pamplona, allowed from 09/23, end with no Moab rollover (reported 10/07). Moab signed a voting agreement at signing.</t>
+          <t>Inferred: live rival when exclusivity with CSC/Pamplona was executed (#44); not reported as told. Its offer, valued by Party B at $21.50 incl. $19.00 cash (#39), lost on certainty (#42).</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>“As a result of such discussions, it was determined that Moab would not rollover any Moab shares in the transaction.” (p. 38)</t>
+          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations” (p. 38)</t>
         </is>
       </c>
       <c r="R47" s="2" t="n"/>
       <c r="S47" s="2" t="n"/>
       <c r="T47" s="3" t="n">
-        <v>41548</v>
+        <v>41541</v>
       </c>
       <c r="U47" s="3" t="n">
-        <v>41542</v>
+        <v>41535</v>
       </c>
       <c r="V47" s="3" t="n">
-        <v>41554</v>
+        <v>41541</v>
       </c>
     </row>
     <row r="48">
@@ -3600,22 +3649,18 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>10/12/2013</t>
+          <t>09/25/2013</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kirkland &amp; Ellis LLP</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Exclusivity changed</t>
+          <t>Adviser</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -3629,31 +3674,29 @@
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Extended to 11:59 p.m. 10/15/2013. CSC/Pamplona asked 10/09; the committee required a termination fee of at most $11 million, agreed 10/11.</t>
+          <t>Outside legal counsel to CSC/Pamplona; first seen acting on 09/25, receiving Goodwin Procter's initial merger-agreement draft.</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed a letter agreement extending exclusivity until 11:59 p.m. ET on October 15, 2013.” (p. 41)</t>
+          <t>“Kirkland &amp; Ellis LLP, outside legal counsel to CSC/Pamplona” (p. 38)</t>
         </is>
       </c>
       <c r="R48" s="2" t="n"/>
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="3" t="n">
-        <v>41559</v>
+        <v>41542</v>
       </c>
       <c r="U48" s="3" t="n">
-        <v>41559</v>
+        <v>41542</v>
       </c>
       <c r="V48" s="3" t="n">
-        <v>41559</v>
+        <v>41542</v>
       </c>
     </row>
     <row r="49">
@@ -3662,7 +3705,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>10/14/2013</t>
+          <t>between 09/25/2013 and 10/07/2013</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3677,7 +3720,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Merger agreement signed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -3698,28 +3741,24 @@
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>$21.25 per share in cash. Pamplona commitment letter ($594m, no financing condition); $11m target fee; $15m reverse fee; MacDonald and Moab voting agreements.</t>
+          <t>Information access after exclusivity: exclusive bidder CSC/Pamplona granted full data-room access (limited earlier, #28) and management access for confirmatory diligence.</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>“Later in the day, on October 14, 2013, the merger agreement was executed, the Pamplona commitment letter was delivered” (p. 41)</t>
-        </is>
-      </c>
-      <c r="R49" s="2" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
+          <t>“CSC and Pamplona were granted full access to the electronic data site and access to certain members of management and conducted confirmatory business and legal due diligence” (p. 38)</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="n"/>
       <c r="S49" s="2" t="n"/>
       <c r="T49" s="3" t="n">
-        <v>41561</v>
+        <v>41542</v>
       </c>
       <c r="U49" s="3" t="n">
-        <v>41561</v>
+        <v>41542</v>
       </c>
       <c r="V49" s="3" t="n">
-        <v>41561</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="50">
@@ -3728,27 +3767,25 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>10/15/2013</t>
+          <t>between 09/25/2013 and 10/07/2013</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray and CSC</t>
+          <t>Moab Partners, L.P. (Moab)</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Merger announced</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
+      <c r="G50" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="2" t="n"/>
@@ -3760,28 +3797,210 @@
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Joint announcement before the market opened. No post-signing competing proposals reported.</t>
+          <t>Rollover resolved, not formed: after Goodwin told Rothenberg on 09/23 that talks could resume, Moab and Pamplona discussed a rollover and determined none (reported 10/07). Moab signed a voting agreement at signing.</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>“Mac-Gray and CSC jointly announced the execution of the merger agreement.” (p. 41)</t>
+          <t>“it was determined that Moab would not rollover any Moab shares in the transaction” (p. 38)</t>
         </is>
       </c>
       <c r="R50" s="2" t="n"/>
       <c r="S50" s="2" t="n"/>
       <c r="T50" s="3" t="n">
+        <v>41548</v>
+      </c>
+      <c r="U50" s="3" t="n">
+        <v>41542</v>
+      </c>
+      <c r="V50" s="3" t="n">
+        <v>41554</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>10/12/2013</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Exclusivity changed</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="n"/>
+      <c r="M51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" s="2" t="n"/>
+      <c r="O51" s="2" t="n"/>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>Extended to 11:59 p.m. ET 10/15/2013 at CSC/Pamplona's request (made by 10/09); committee required a Mac-Gray termination fee of at most $11m, which CSC/Pamplona accepted on 10/11.</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>“CSC, Pamplona and Mac-Gray executed a letter agreement extending exclusivity until 11:59 p.m. ET on October 15, 2013” (p. 41)</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="n"/>
+      <c r="S51" s="2" t="n"/>
+      <c r="T51" s="3" t="n">
+        <v>41559</v>
+      </c>
+      <c r="U51" s="3" t="n">
+        <v>41559</v>
+      </c>
+      <c r="V51" s="3" t="n">
+        <v>41559</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>10/14/2013</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Merger agreement signed</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="n"/>
+      <c r="M52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="2" t="n"/>
+      <c r="O52" s="2" t="n"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>$21.25 per share in cash; buyers Spin Holdco (Parent), CSC ServiceWorks Holdings and CSC. Pamplona commitment letter $594m; Pamplona liability cap $50m; Mac-Gray fee $11m; CSC reverse fee $15m. Moab and MacDonald voting agreements effective. BofA fairness opinion same day.</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>“Later in the day, on October 14, 2013, the merger agreement was executed, the Pamplona commitment letter was delivered” (p. 41)</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="n"/>
+      <c r="S52" s="2" t="n"/>
+      <c r="T52" s="3" t="n">
+        <v>41561</v>
+      </c>
+      <c r="U52" s="3" t="n">
+        <v>41561</v>
+      </c>
+      <c r="V52" s="3" t="n">
+        <v>41561</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>10/15/2013</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Merger announced</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="n"/>
+      <c r="M53" s="2" t="n"/>
+      <c r="N53" s="2" t="n"/>
+      <c r="O53" s="2" t="n"/>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>Joint announcement by Mac-Gray and CSC before the market opened. Ref: $14.72 close 10/11/2013; about 44% premium (p. 5).</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>“before the U.S. stock markets opened, Mac-Gray and CSC jointly announced the execution of the merger agreement” (p. 41)</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="n"/>
+      <c r="S53" s="2" t="n"/>
+      <c r="T53" s="3" t="n">
         <v>41562</v>
       </c>
-      <c r="U50" s="3" t="n">
+      <c r="U53" s="3" t="n">
         <v>41562</v>
       </c>
-      <c r="V50" s="3" t="n">
+      <c r="V53" s="3" t="n">
         <v>41562</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V50"/>
+  <autoFilter ref="A1:V53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3803,8 +4022,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3867,16 +4086,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>41451</v>
+        <v>41449</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BofA outreach to 50 parties after the 06/24 decision; NDA signers asked for preliminary IOIs</t>
+          <t>Special Committee's 06/24 decision executed: BofA outreach to 50 parties; confidentiality signers asked for preliminary indications</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>20: 2 strategic (CSC/Pamplona; Party A via its standing 06/21 proposal, NDA only on 08/05) and 18 financial (Party B, Party C, 16 unnamed NDA signers)</t>
+          <t>20 entered: 2 strategic (CSC/Pamplona; Party A via its standing round-0 proposal, no NDA until 08/05) and 18 financial (Party B, Party C, 16 unnamed signers, dates unknown)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -3896,12 +4115,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>3: CSC/Pamplona, Party B, Party C (oral, then written); Party A's round-0 proposal also reviewed</t>
+          <t>3: CSC/Pamplona, Party B, Party C (plus Party A's 06/21 round-0 proposal, reviewed 07/25)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>four advanced (Party A, Party B, Party C, CSC/Pamplona); 16 financial signers out</t>
+          <t>four advanced (Party A, Party B, Party C, CSC/Pamplona); 16 other financial signers out</t>
         </is>
       </c>
     </row>
@@ -3917,7 +4136,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>committee advanced four, set up management meetings and staged data-room access, then asked for revised IOIs</t>
+          <t>committee advanced four to management meetings and staged diligence, then asked for revised written proposals</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -3942,12 +4161,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>4: CSC/Pamplona, Party B, Party A, Party C</t>
+          <t>4: CSC/Pamplona and Party B (09/09), Party A and Party C (09/10)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>all four asked for final IOIs; none out</t>
+          <t>all four asked for final indications on 09/11</t>
         </is>
       </c>
     </row>
@@ -3963,7 +4182,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>committee asked all four for final IOIs by 09/18, with short exclusivity for one</t>
+          <t>committee asked all four for final indications, holding out short exclusivity</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -3988,12 +4207,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>3: CSC/Pamplona ($20.75, raised to $21.25 on 09/21), Party B ($21.50 package), Party A (reaffirmed $18.00-$19.00); Party C did not submit</t>
+          <t>3: CSC/Pamplona, Party B, Party A (reaffirmed best and final); Party C did not submit</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona chosen 09/19, exclusivity 09/24, signing 10/14; Party A and Party B dropped, Party C out</t>
+          <t>CSC/Pamplona selected 09/19 and raised to $21.25 on 09/21; exclusivity 09/24 (Party A, Party B out); signing 10/14</t>
         </is>
       </c>
     </row>
@@ -4009,16 +4228,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4066,27 +4285,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Process and round map: one process, three rounds opening at the outreach (06/24-06/28), the 07/25 advancement of four, and the 09/11 final request?</t>
+          <t>Process and round map: one process with three rounds (outreach 06/24; four advanced 07/25; final indications 09/11)?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Yes, as recorded.</t>
+          <t>Yes. One process; round 0 holds Party A's 06/21 proposal; R1 opens with the outreach launched 06/24; R2 on 07/25; R3 on 09/11 (announced final).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>07/25: target picked who advanced and opened a staged information stage for revised IOIs (pp. 33-34). 09/11: first request for final IOIs (p. 36).</t>
+          <t>Gaps of two months or more: 04/08/2013 (BofA–Party A call) to 06/21/2013 (Party A proposal), 74 days, both dates certain; no other. C7: (a) fails, since Party A was kept in view (05/09 report; named in 06/24 outreach); (b) fails, gap under three months; (c) met (05/09, 06/24). The 2011–2012 CSC talks had Mac-Gray as buyer (pp. 27–31).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>8, 9, 23, 25-27, 34</t>
+          <t>#8, #10, #25, #36, #27, #28</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>If round 2 opened with the 08/27 letter, #23, #25 and #26 move to round 1. Bid rounds are unchanged.</t>
+          <t>Most plausible alternative: R2 opens with the 08/27 letter, not the 07/25 decision; #25 would move and #27, #28 would fall in R1. R1 opening date alternatives (06/24 decision vs first calls by 06/28) do not move any bid.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -4099,27 +4318,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Deadline outcomes: 07/23 Late bids accepted; 09/09 Late bids accepted; 09/18 Enforced?</t>
+          <t>Deadline outcomes: R1 (07/23) and R2 (09/09) Late bids accepted; R3 (09/18) Enforced?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Yes, as recorded.</t>
+          <t>Yes. R1: Party B and Party C bid 07/24 (Party C again 07/25) after receiving the 07/23 date, and all were reviewed 07/25. R2: Party A and Party C bid 09/10 and were reviewed 09/11. R3: committee selected CSC/Pamplona 09/19 on the bids in hand.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>B and C bid 07/24, reviewed 07/25 (p. 33). A and C bid 09/10, reviewed 09/11 (p. 35). The 09/19 selection used bids in hand (p. 37).</t>
+          <t>Due dates pp. 32, 35, 36; bids pp. 33–36; selection p. 37. The 07/23 instruction went to confidentiality signers, including Party B and Party C, whose agreements predate it (p. 32).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>19, 21, 22, 30, 31, 32, 39</t>
+          <t>#16, #21, #22, #23, #26, #29, #32, #33, #34, #41</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>If one-day slips count as on time, 07/23 and 09/09 become Enforced. Live counts are unchanged.</t>
+          <t>If the one-day slippages were treated as immaterial, R1 and R2 would read Passed without action or Enforced; neither changes any row, but both would overstate enforcement.</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -4132,27 +4351,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Were all 16 unnamed financial NDA signers eligible at the 07/23 due date?</t>
+          <t>Are the 09/18 answers to the request for 'final indications of interest' and CSC/Pamplona's 09/21 $21.25 'last and best offer' Formal?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Yes: Did not submit at 07/23 (inferred).</t>
+          <t>Formal (C13 rule 2): the 09/11 request was an announced final solicitation. No markup was delivered; Goodwin sent the first draft only on 09/25. Party A expressly called its range best and final.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>The 20 NDAs were signed 'over the next two months', undated (p. 32). On 07/25 only four bidders were named (p. 34).</t>
+          <t>The request for final indications came with the prospect of exclusivity (p. 36); CSC/Pamplona called $21.25 its 'last and best offer' (p. 37). Evidence is thin because no documents accompanied the bids.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>13, 20</t>
+          <t>#37, #38, #39, #43</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Late signers would instead be Dropped by target on 07/25 or later. The live count after 07/25 stays four.</t>
+          <t>If Informal, the winner reaches signing with no Formal row, and C12 would add a Bid reaffirmed for CSC/Pamplona at 10/07 (Kirkland's revised merger-agreement draft, p. 39), at $21.25 carried from #43, Conditions Unclear.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -4165,27 +4384,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Are the round-3 bids Formal, though called 'indications of interest' with no markup before exclusivity?</t>
+          <t>The 16 unnamed financial confidentiality signers: are they (and Party B, Party C) within the 35 financial contacts, and did they leave by the 07/25 advancement (Dropped by target) or by the 07/23 due date (Did not submit)?</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Yes, Formal (C13 rule 2): they answer the 09/11 final request as asked.</t>
+          <t>Keep: within the 35; Dropped by target by 07/25, inferred, Count 16.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Final request p. 36. CSC/Pamplona's $21.25 is a 'last and best offer' (p. 37). Kirkland returned a merger agreement draft on 10/07 (p. 39).</t>
+          <t>The filing gives 20 signers (2 strategic, 18 financial) over two months but no dates for the 16, so it cannot show they had signed before 07/23; the four-bidder set advanced on 07/25 is complete (pp. 32–34).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>35, 36, 37, 41</t>
+          <t>#12, #13, #24</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>If Informal: add a CSC/Pamplona Bid reaffirmed at $21.25 on 10/07 (returned draft); Party A and Party B final bids become Informal.</t>
+          <t>Did not submit by 07/23 would change the exit label and round-1 non-submission count, not the live count. If some signed after 07/25, their exit would be by 08/27 (letters to four only).</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -4198,66 +4417,33 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>How should Party B's 09/18 cash-plus-options package be priced?</t>
+          <t>Party B's 09/18 price: record $21.50 (its own value incl. options) or $19.00 cash?</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>$21.50 (Party B's own valuation), All cash = No; the Note gives $19.00 cash + options valued at $2.50.</t>
+          <t>$21.50 in both price cells, All cash = No, with $19.00 cash and $2.50 option value in the Note.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>'valued at $21.50 per share, including $19.00 of cash'; options vest on five-year targets (p. 36).</t>
+          <t>C15: a stated per-share package value is the total offer value. Party B valued the options at $2.50; the committee questioned that value (pp. 36–37).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>37, 44</t>
+          <t>#39</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Cash-only $19.00 would rank Party B below CSC/Pamplona's $20.75.</t>
+          <t>Using $19.00 would make Party B's final bid lower than CSC/Pamplona's $20.75, changing the reading of why it lost and the ranking of final bids.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Is the winner CSC/Pamplona Strategic or Mixed?</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Strategic: sponsor-owned laundry operator; Pamplona provides equity.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>The filing calls CSC/Pamplona a strategic bidder (pp. 32, 34). Parent is a CSC subsidiary (p. 26). Pamplona commits $594m (p. 59).</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>10, 17, 18, 28, 35, 41, 42, 47, 48</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Mixed if Pamplona is a co-bidder: it signed the NDA and exclusivity and has liability up to $50m. The strategic/financial split would shift.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4268,11 +4454,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4307,7 +4493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CSC ServiceWorks, Inc. (via Spin Holdco Inc. and CSC Fenway, Inc.; with CSC ServiceWorks Holdings, Inc.), a portfolio company of Pamplona Capital; funded by Pamplona Capital Partners III, L.P.</t>
+          <t>CSC ServiceWorks, Inc., through Spin Holdco Inc. (Parent), CSC ServiceWorks Holdings, Inc. and CSC Fenway, Inc.; CSC is owned by Pamplona Capital Partners III, L.P., which committed the equity (the filing calls the bidder "CSC/Pamplona")</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4505,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Strategic (sponsor-owned operating company)</t>
+          <t>Strategic: laundry facilities operator owned by a private equity fund (Pamplona), which funds the deal; the filing calls CSC/Pamplona a strategic bidder (p. 32)</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4517,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>$21.25 per share in cash</t>
+          <t>$21.25 per share in cash; equity funded by a $594m Pamplona commitment letter; no financing condition</t>
         </is>
       </c>
     </row>
@@ -4341,8 +4527,10 @@
           <t>Merger agreement signed</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
-        <v>41561</v>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>10/14/2013</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4351,8 +4539,10 @@
           <t>Merger announced</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>41562</v>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>10/15/2013</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -4363,7 +4553,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>DEFM14A, 12/04/2013</t>
+          <t>DEFM14A (definitive proxy statement), 12/04/2013</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4565,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>27-41</t>
+          <t>pp. 27–41</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4577,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>target-led</t>
+          <t>target-led: Board authorized BofA to explore opportunities (04/05/2013) and BofA sounded out Party A (04/08); Party A then made an unsolicited proposal (06/21) before the organized outreach. An activist (Moab) won board seats on 05/30/2013 but is not reported pressing for a sale.</t>
         </is>
       </c>
     </row>
@@ -4397,84 +4587,98 @@
           <t>Number of processes</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>1</v>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Auction screen</t>
+          <t>Earlier approaches</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Met: 20 confidentiality agreements (2 strategic, 18 financial)</t>
+          <t>Winter 2011 into 2012: talks between Mac-Gray and CSC about Mac-Gray acquiring CSC (Mac-Gray as buyer; BofA engaged 10/23/2012); CSC was instead sold to Pamplona in May 2013. Undated discussions with other industry participants. None was a sale of Mac-Gray.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Whole-company bids</t>
+          <t>Auction screen</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Met (process 1): 20 parties. The filing counts 20 potential bidders (parties) signing confidentiality agreements: 2 strategic, 18 financial; CSC and Pamplona counted as one. No post-signing additions.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Currency and units of bid prices</t>
+          <t>Whole-company bids</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>US dollars per share; Party B's 09/18 bid is $19.00 cash plus options it valued at $2.50</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Target financial advisers</t>
+          <t>Currency and units of bid prices</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>BofA Merrill Lynch (sole)</t>
+          <t>US dollars per share. Party B's 09/18 bid mixed $19.00 cash with options it valued at $2.50 per share (Q5); all others all cash.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Target legal advisers</t>
+          <t>Target financial advisers</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Goodwin Procter LLP</t>
+          <t>BofA Merrill Lynch (Merrill Lynch, Pierce, Fenner &amp; Smith Incorporated), sole financial adviser; engaged 05/31/2013 after its 2011–2012 mandate was ended 05/15/2013</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Target legal advisers</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Goodwin Procter LLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Mac-Gray, the second-largest US laundry facilities management contractor, had BofA Merrill Lynch sound out strategic rival Party A in April 2013; Party A made an unsolicited $17.00-$19.00 proposal on June 21. On June 24 a new Special Committee decided to consider a sale, and BofA contacted 50 parties (15 strategic, 35 financial), 20 of which signed confidentiality agreements. Preliminary indications from CSC/Pamplona ($18.50), Party B ($17.00-$18.00) and Party C ($15.00-$17.00, then $16.00-$16.50) led the committee to advance four bidders, including Party A, to management meetings and staged data-room access, with less customer data shown to strategic bidders. Revised indications on September 9-10 ranged from $16.00 to $19.50. A request for final indications by September 18 drew $20.75 from CSC/Pamplona, a $21.50 cash-plus-options package from Party B, Party A's unchanged $18.00-$19.00 and nothing from Party C. The committee preferred CSC/Pamplona's fully Pamplona-funded offer for its certainty, asked for $21.25, and signed exclusivity on September 24 once CSC/Pamplona agreed. After one extension of exclusivity, the merger agreement was signed on October 14, 2013 at $21.25 per share in cash and announced on October 15.</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>In spring 2013 Mac-Gray's board, with BofA Merrill Lynch, began exploring a sale; Party A made an unsolicited $17–19 all-cash proposal on 06/21/2013. A Special Committee then had BofA approach 50 parties, and 20 (2 strategic, 18 financial) signed confidentiality agreements. Preliminary indications from CSC/Pamplona ($18.50), Party B ($17–18) and Party C ($15–17, then $16–16.50) led the committee to advance four bidders, including Party A, to management meetings and staged diligence. Revised proposals (09/09–09/10) ranged from $16–17 to $19.50, and final indications on 09/18 brought CSC/Pamplona to $20.75 and Party B to a cash-and-options package it valued at $21.50; Party A stood at $18–19 and Party C dropped out. The committee preferred CSC/Pamplona's fully funded offer, obtained $21.25 in exchange for exclusivity (09/24), and signed on 10/14/2013 after negotiating fees and Pamplona's liability.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate Opus extraction workspace and editable cockpit
Record the approved v1.13.2 instruction, nine-deal Opus set, immutable workbook versions, and review evidence. Checkpoint the editable cockpit and pipeline integrity repairs.

Retire Grok and Sol comparison results and their catalog dependencies. Preserve the Astra experiment as a historical side note only. Refresh the handoff and record exact deletion, preservation, and verification evidence.

Validation: 99 Python unit tests, 11 HTTP acceptance tests, 3 frontend tests, production build, and nine-deal catalog and live-document checks passed.
</commit_message>
<xml_diff>
--- a/extraction/mac-gray.xlsx
+++ b/extraction/mac-gray.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal facts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rounds'!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal facts'!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,10 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
-    <numFmt numFmtId="166" formatCode="$0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -72,7 +71,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -440,14 +439,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V53"/>
+  <dimension ref="A1:V55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
@@ -456,12 +455,12 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="60" customWidth="1" min="16" max="16"/>
-    <col width="55" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
@@ -585,7 +584,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>04/05/2013</t>
+          <t>10/23/2012</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -615,24 +614,24 @@
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray's financial adviser, first seen acting in the sale context: Board authorized management to work with it to explore transactions, incl. with Party A. Engaged 10/23/2012 for the 2011–2012 Discussions (Mac-Gray's possible purchase of CSC).</t>
+          <t>Mac-Gray's financial adviser, first engaged for the 2011-2012 Discussions (Mac-Gray's possible acquisition of CSC). The filing does not say under which engagement BofA made the 04/08/2013 call to Party A.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>“authorized Mac-Gray management to work with BofA Merrill Lynch to explore transactional opportunities that might be available to Mac-Gray” (p. 27)</t>
+          <t>In connection with Mac-Gray's consideration of a possible acquisition of CSC, which we refer to as the 2011-2012 Discussions, Mac-Gray engaged BofA Merrill Lynch on October 23, 2012. (p. 27)</t>
         </is>
       </c>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="3" t="n">
-        <v>41369</v>
+        <v>41205</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>41369</v>
+        <v>41205</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>41369</v>
+        <v>41205</v>
       </c>
     </row>
     <row r="3">
@@ -677,15 +676,19 @@
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>BofA, as instructed by the Board, called Party A (a laundry facilities management company) about a possible combination; Party A said it might consider one. First contact with Party A.</t>
+          <t>BofA, instructed by the board (04/05/2013 authorization to explore transactional opportunities, including with Party A), called Party A about a possible business combination; Party A said it might consider one. First contact with Party A.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>“the representative of Party A indicated that Party A might consider a business combination with Mac-Gray” (p. 27)</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="n"/>
+          <t>representatives of BofA Merrill Lynch, as instructed by the Board, telephoned a representative of Party A to discuss generally a possible business combination between Party A and Mac-Gray (p. 27)</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="n"/>
       <c r="T3" s="3" t="n">
         <v>41372</v>
@@ -733,12 +736,12 @@
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray's outside legal counsel; first seen acting at the 05/09 Board meeting. Later also advised the Special Committee.</t>
+          <t>Mac-Gray's outside legal counsel; earliest reported acting at the 05/09/2013 board meeting, where the board formed the Transaction Committee to pick a financial adviser for a strategic-alternatives review.</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>“Goodwin Procter LLP, outside legal counsel to Mac-Gray” (p. 27)</t>
+          <t>representatives from BofA Merrill Lynch and Goodwin Procter LLP, outside legal counsel to Mac-Gray, were also in attendance for all or portions of the meeting (p. 27)</t>
         </is>
       </c>
       <c r="R4" s="2" t="n"/>
@@ -759,18 +762,18 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>05/09/2013</t>
+          <t>05/15/2013</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
+          <t>BofA Merrill Lynch</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Target sale decision</t>
+          <t>Adviser ended</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -789,24 +792,24 @@
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Board discussed a possible sale process and its risks (leaks, disclosure to competitors); formed a Transaction Committee (Bullock, Daoust) to recommend a financial adviser for a strategic-alternatives review incl. a sale. Qualification: sale-process decision deferred.</t>
+          <t>Mac-Gray terminated BofA's 2011-2012 Discussions engagement (decided by the Transaction Committee 05/14/2013) because BofA was being invited to pitch for the new strategic-alternatives mandate and the CSC sale process had ended.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>“The Board concluded that it would discuss the review of strategic alternatives, including engaging in a potential sale process, at its next meeting” (p. 28)</t>
+          <t>On May 15, 2013, Mac-Gray sent a letter to BofA Merrill Lynch terminating their engagement in connection with the 2011-2012 Discussions. (p. 29)</t>
         </is>
       </c>
       <c r="R5" s="2" t="n"/>
       <c r="S5" s="2" t="n"/>
       <c r="T5" s="3" t="n">
-        <v>41403</v>
+        <v>41409</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>41403</v>
+        <v>41409</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>41403</v>
+        <v>41409</v>
       </c>
     </row>
     <row r="6">
@@ -815,7 +818,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>05/15/2013</t>
+          <t>05/30/2013</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -826,7 +829,7 @@
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Adviser ended</t>
+          <t>Adviser</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -845,24 +848,24 @@
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray terminated BofA's 2011–2012 Discussions engagement letter (Transaction Committee decision 05/14), because BofA was to pitch for the new sale mandate and the CSC sale had ended.</t>
+          <t>Board approved engaging BofA as Mac-Gray's financial adviser for the strategic-alternatives review, including a potential sale, after a three-bank pitch; engagement letter signed 05/31/2013 barred BofA from financing buyers without consent.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>“Mac-Gray sent a letter to BofA Merrill Lynch terminating their engagement in connection with the 2011-2012 Discussions” (p. 29)</t>
+          <t>Based on the recommendation of the Transaction Committee, the Board unanimously approved the engagement of BofA Merrill Lynch on the terms discussed at this meeting. (p. 29)</t>
         </is>
       </c>
       <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="3" t="n">
-        <v>41409</v>
+        <v>41424</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>41409</v>
+        <v>41424</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>41409</v>
+        <v>41424</v>
       </c>
     </row>
     <row r="7">
@@ -876,13 +879,13 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>BofA Merrill Lynch</t>
+          <t>Moab Partners, L.P. (with affiliates)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Activist</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -901,12 +904,12 @@
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Re-engaged as Mac-Gray's (sole) financial adviser for the strategic-alternatives review incl. a sale, chosen over two other banks (pitches 05/22, 05/29). Letter signed 05/31 bars it from financing buyers without consent. Fee about $8.1m (p. 51).</t>
+          <t>Moab won a proxy contest: its nominees Rothenberg (Moab's co-founder and General Partner) and Hyman replaced two incumbents at the annual meeting. Moab held about 9% (as of 06/12/2013). The filing does not say Moab pressed for a sale.</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>“the Board unanimously approved the engagement of BofA Merrill Lynch on the terms discussed at this meeting” (p. 29)</t>
+          <t>the Mac-Gray stockholders elected as directors Michael M. Rothenberg and James E. Hyman, candidates nominated by Mac-Gray's stockholder, Moab Partners, L.P. and certain of its affiliates (p. 29)</t>
         </is>
       </c>
       <c r="R7" s="2" t="n"/>
@@ -927,18 +930,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>05/30/2013</t>
+          <t>06/21/2013</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Moab Partners, L.P. (Moab)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Activist</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -947,34 +954,56 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
+      <c r="H8" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Moab (about 9% holder, per 06/12) won a proxy contest: its nominees Rothenberg (Moab general partner) and Hyman joined the Board. Moab later sought a possible equity rollover (#18, #49); Rothenberg excluded from sale deliberations.</t>
+          <t>Conditions unclear: the filing reports no financing or diligence terms. Unsolicited written proposal to the board, before any outreach or NDA; the Special Committee expected Party A to raise it after diligence.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>“the Mac-Gray stockholders elected as directors Michael M. Rothenberg and James E. Hyman, candidates nominated by Mac-Gray's stockholder, Moab Partners, L.P.” (p. 29)</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="n"/>
+          <t>Party A submitted an unsolicited proposal to the Mac-Gray Board of Directors offering to purchase Mac-Gray for an all-cash purchase price of $17.00 to $19.00 per share (p. 30)</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="3" t="n">
-        <v>41424</v>
+        <v>41446</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>41424</v>
+        <v>41446</v>
       </c>
       <c r="V8" s="3" t="n">
-        <v>41424</v>
+        <v>41446</v>
       </c>
     </row>
     <row r="9">
@@ -983,22 +1012,18 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>06/21/2013</t>
+          <t>06/24/2013</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Target sale decision</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1007,56 +1032,34 @@
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: no confidentiality agreement or diligence until 08/05 (#27). Unsolicited written proposal to the Board; Party A enters the process. Financing not stated.</t>
+          <t>Board formed a six-member Special Committee (MacDonald and Rothenberg excluded). The Committee concluded it should consider a potential sale, to be weighed against remaining stand-alone; buybacks and a special dividend were rejected.</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>“Party A submitted an unsolicited proposal to the Mac-Gray Board of Directors offering to purchase Mac-Gray for an all-cash purchase price of $17.00 to $19.00 per share” (p. 30)</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+          <t>the Special Committee concluded that it would be in the best interests of stockholders to consider a potential sale of Mac-Gray (p. 31)</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="n"/>
       <c r="S9" s="2" t="n"/>
       <c r="T9" s="3" t="n">
-        <v>41446</v>
+        <v>41449</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>41446</v>
+        <v>41449</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>41446</v>
+        <v>41449</v>
       </c>
     </row>
     <row r="10">
@@ -1076,14 +1079,14 @@
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Target sale decision</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -1095,15 +1098,19 @@
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Board excluded CEO MacDonald and Rothenberg (possible rollover partners) and formed a six-member independent Special Committee. Committee decided to consider a sale against the stand-alone plan and to approach 50 parties (15 strategic, 35 financial). Projections presented.</t>
+          <t>Special Committee decided to approach 50 parties (15 strategic, 35 financial, including CSC/Pamplona and Party A); BofA began outreach within days (first NDA 06/28/2013). NDA signers received an informational package and were asked for preliminary indications by 07/23/2013.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee concluded that it would be in the best interests of stockholders to consider a potential sale of Mac-Gray” (p. 31)</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="n"/>
+          <t>BofA Merrill Lynch contacted the strategic and financial parties identified at the June 24th Special Committee meeting (p. 32)</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="n"/>
       <c r="T10" s="3" t="n">
         <v>41449</v>
@@ -1121,18 +1128,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>06/24/2013–06/28/2013 (outreach begins)</t>
+          <t>during the weeks after 06/24/2013</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n"/>
+          <t>13 other potential strategic buyers</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -1146,24 +1157,22 @@
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="M11" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>BofA began contacting the 50 parties chosen on 06/24 over the following weeks; calls with Party A and Pamplona reported by 06/28. Confidentiality signers received an information package and a request for preliminary indications (#16).</t>
+          <t>Target outreach by BofA. The filing's total of 15 strategic parties approached includes CSC/Pamplona (own row) and Party A (first contacted 04/08/2013, #2; BofA spoke to it again by 06/28/2013). None of these 13 signed an NDA (only two strategic signers).</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>“BofA Merrill Lynch contacted the strategic and financial parties identified at the June 24th Special Committee meeting” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+          <t>and Party A, to solicit potential interest in a transaction with Mac-Gray, 15 of which were potential strategic buyers and 35 of which were potential financial buyers (p. 32)</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="n"/>
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="3" t="n">
         <v>41449</v>
@@ -1171,9 +1180,7 @@
       <c r="U11" s="3" t="n">
         <v>41449</v>
       </c>
-      <c r="V11" s="3" t="n">
-        <v>41453</v>
-      </c>
+      <c r="V11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1181,17 +1188,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>during the several weeks after 06/24/2013</t>
+          <t>during the weeks after 06/24/2013</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>13 other strategic parties</t>
+          <t>35 potential financial buyers, including private equity firms</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1211,18 +1218,18 @@
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Target outreach. Total 50 = 15 strategic + 35 financial, incl. Party A (first contacted 04/08, #2; spoke again 06/28, citing synergies and financing sources) and CSC/Pamplona (#14): 15 − 2 = 13. Responses not reported.</t>
+          <t>Target outreach by BofA. Includes Party B and Party C. 18 of the 35 later signed NDAs; the rest did not.</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>“50 parties, including CSC and Pamplona, who together we refer to as CSC/Pamplona, and Party A, to solicit potential interest in a transaction with Mac-Gray” (p. 32)</t>
+          <t>35 of which were potential financial buyers, including private equity firms (p. 32)</t>
         </is>
       </c>
       <c r="R12" s="2" t="n"/>
@@ -1241,17 +1248,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>during the several weeks after 06/24/2013</t>
+          <t>by 06/28/2013</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>35 financial parties (incl. Party B, Party C)</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1271,33 +1278,31 @@
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Target outreach to 35 financial buyers, incl. private equity firms. Party B and Party C assumed to be among them (filing does not say so expressly; Q4). Rows reconcile to 50: 35 + 13 (#11) + CSC/Pamplona + Party A.</t>
+          <t>Target outreach: BofA, as instructed, spoke with Pamplona, which was interested in an acquisition by its portfolio company CSC and said diligence would be minimal. In the same report, Party A cited synergies and was speaking to financing sources.</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>“15 of which were potential strategic buyers and 35 of which were potential financial buyers, including private equity firms” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
+          <t>BofA Merrill Lynch also reported that they had spoken with representatives of Pamplona, as instructed by the Special Committee, who expressed interest in a transaction (p. 32)</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="n"/>
       <c r="S13" s="2" t="n"/>
       <c r="T13" s="3" t="n">
-        <v>41449</v>
+        <v>41451</v>
       </c>
       <c r="U13" s="3" t="n">
         <v>41449</v>
       </c>
-      <c r="V13" s="2" t="n"/>
+      <c r="V13" s="3" t="n">
+        <v>41453</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1305,22 +1310,18 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>06/24/2013–08/24/2013 (over the next two months)</t>
+          <t>by 06/28/2013</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>16 other financial NDA signers</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Deadline set</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -1334,35 +1335,37 @@
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n">
-        <v>16</v>
-      </c>
+      <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Filing total: 20 signers over two months = 2 strategic (Party A #27, CSC/Pamplona #19) + 18 financial incl. Party B (#15), Party C (#17); residual 18 − 2 = 16. Dates not reported. Standstills had sunset provisions. Each received the information package.</t>
+          <t>NDA signers were told to submit preliminary indications by 07/23/2013 (valuation, financing, conditions, diligence focus). Date inferred: the instruction came with the informational package, and the first package reported went to Party B on 06/28/2013.</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>“a total of 20 potential bidders, including two strategic bidders (Party A and CSC/Pamplona) and 18 financial bidders (including Party B and Party C), entered into confidentiality agreements” (p. 32)</t>
+          <t>furnished an informational package for the purpose of providing potential bidders with data to formulate a preliminary indication of interest, which they were instructed to submit by July 23, 2013 (p. 32)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
       <c r="T14" s="3" t="n">
-        <v>41449</v>
+        <v>41453</v>
       </c>
       <c r="U14" s="3" t="n">
         <v>41449</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>41510</v>
+        <v>41453</v>
       </c>
     </row>
     <row r="15">
@@ -1371,22 +1374,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>by 06/28/2013</t>
+          <t>06/28/2013</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
+          <t>Party B</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1407,21 +1410,21 @@
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>BofA, as instructed, called Pamplona, which was interested incl. in an acquisition by its portfolio company CSC; said diligence would be minimal given its familiarity. One bidder unit; filing classes it strategic.</t>
+          <t>Confidentiality and standstill agreement with a sunset clause; Party B received the informational package. Entry.</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>“Pamplona emphasized that business and legal due diligence would be minimal given its familiarity with Mac-Gray and the industry generally” (p. 32)</t>
+          <t>Later on June 28, 2013, Party B, entered into a confidentiality and standstill agreement with Mac-Gray (p. 32)</t>
         </is>
       </c>
       <c r="R15" s="2" t="n"/>
       <c r="S15" s="2" t="n"/>
       <c r="T15" s="3" t="n">
-        <v>41451</v>
+        <v>41453</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>41449</v>
+        <v>41453</v>
       </c>
       <c r="V15" s="3" t="n">
         <v>41453</v>
@@ -1433,12 +1436,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>06/28/2013</t>
+          <t>06/30/2013</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>Party C</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1469,24 +1472,24 @@
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Enters: confidentiality and standstill agreement; received the information package for a preliminary indication. Financial bidder (p. 32).</t>
+          <t>Confidentiality and standstill agreement; Party C received the informational package. Entry.</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>“Party B, entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 32)</t>
+          <t>On June 30, 2013, Party C entered into a confidentiality and standstill agreement with Mac-Gray (p. 32)</t>
         </is>
       </c>
       <c r="R16" s="2" t="n"/>
       <c r="S16" s="2" t="n"/>
       <c r="T16" s="3" t="n">
-        <v>41453</v>
+        <v>41455</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>41453</v>
+        <v>41455</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>41453</v>
+        <v>41455</v>
       </c>
     </row>
     <row r="17">
@@ -1495,18 +1498,18 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>06/28/2013 (with information packages)</t>
+          <t>07/03/2013</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
+          <t>Moab Partners (Rothenberg) and CSC/Pamplona</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Deadline set</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -1522,35 +1525,27 @@
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Preliminary indications due 07/23/2013, to address valuation, financing, conditions and diligence focus. The instruction came with each signer's information package; dated at the first reported package (Party B, #15).</t>
+          <t>Rollover approach: Rothenberg told Goodwin that he had discussed a possible Moab equity rollover with Pamplona, and that Pamplona would ask for its NDA to let it share its bid with Moab, with Moab dealing only with CSC/Pamplona.</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>“which they were instructed to submit by July 23, 2013” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+          <t>Pamplona would be requesting that any confidentiality agreement CSC/Pamplona execute with Mac-Gray permit CSC and Pamplona to discuss their bid and evaluation material with Moab (p. 32)</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="n"/>
       <c r="S17" s="2" t="n"/>
       <c r="T17" s="3" t="n">
-        <v>41453</v>
+        <v>41458</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>41453</v>
+        <v>41458</v>
       </c>
       <c r="V17" s="3" t="n">
-        <v>41453</v>
+        <v>41458</v>
       </c>
     </row>
     <row r="18">
@@ -1559,22 +1554,18 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>06/30/2013</t>
+          <t>07/06/2013</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Mac-Gray</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1588,31 +1579,29 @@
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Enters: confidentiality and standstill agreement; received the information package. Financial bidder (p. 32).</t>
+          <t>Special Committee refused the Moab–CSC/Pamplona exclusive rollover arrangement, keeping Moab's stake available to all bidders; told CSC/Pamplona and Rothenberg that rollover talks with anyone were premature but would be allowed later.</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>“Party C entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 32)</t>
+          <t>the Special Committee decided to deny the exclusivity request at this stage of the process so that the potential equity rollover of Moab's shares could be available (p. 33)</t>
         </is>
       </c>
       <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="3" t="n">
-        <v>41455</v>
+        <v>41461</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>41455</v>
+        <v>41461</v>
       </c>
       <c r="V18" s="3" t="n">
-        <v>41455</v>
+        <v>41461</v>
       </c>
     </row>
     <row r="19">
@@ -1621,18 +1610,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>07/06/2013</t>
+          <t>07/11/2013</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="n"/>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -1646,29 +1639,31 @@
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
+      <c r="M19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Refused rollover partnership: on 07/03 Rothenberg said Pamplona would seek confidentiality terms letting CSC/Pamplona share its bid and data with Moab, Moab dealing exclusively with them. Special Committee refused; rollover talks premature with anyone, allowed later.</t>
+          <t>Confidentiality and standstill agreement (a letter agreement among Pamplona Capital Management LLC, Parent and Mac-Gray, per merger agreement s.6.17, Annex A); informational package provided. Entry. Party A's NDA talks stalled over non-solicitation terms 07/11–07/23.</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee decided to deny the exclusivity request at this stage of the process” (p. 33)</t>
+          <t>On July 11, 2013, CSC/Pamplona entered into a confidentiality and standstill agreement with Mac-Gray (p. 33)</t>
         </is>
       </c>
       <c r="R19" s="2" t="n"/>
       <c r="S19" s="2" t="n"/>
       <c r="T19" s="3" t="n">
-        <v>41461</v>
+        <v>41466</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>41461</v>
+        <v>41466</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>41461</v>
+        <v>41466</v>
       </c>
     </row>
     <row r="20">
@@ -1677,17 +1672,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>07/11/2013</t>
+          <t>06/24/2013 to about 08/24/2013 ("over the next two months")</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
+          <t>16 other financial NDA signers</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1707,30 +1702,34 @@
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Enters: confidentiality and standstill agreement signed by CSC/Pamplona; received the information package. CSC is a laundry operator owned by Pamplona (private equity fund).</t>
+          <t>Count: 16 = 20 NDA signers (2 strategic, 18 financial) minus the individually recorded Party A, CSC/Pamplona, Party B and Party C. Signing dates not reported; some may have signed after 07/23/2013. Sort date moved to 07/23/2013 to precede the inferred exit.</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona entered into a confidentiality and standstill agreement with Mac-Gray and were provided with an informational package” (p. 33)</t>
-        </is>
-      </c>
-      <c r="R20" s="2" t="n"/>
+          <t>a total of 20 potential bidders, including two strategic bidders (Party A and CSC/Pamplona) and 18 financial bidders (including Party B and Party C), entered into confidentiality agreements (p. 32)</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
       <c r="S20" s="2" t="n"/>
       <c r="T20" s="3" t="n">
-        <v>41466</v>
+        <v>41478</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>41466</v>
+        <v>41449</v>
       </c>
       <c r="V20" s="3" t="n">
-        <v>41466</v>
+        <v>41510</v>
       </c>
     </row>
     <row r="21">
@@ -1791,12 +1790,12 @@
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: management presentation 08/12; limited data-room access, customer data reserved (#28). Preliminary indication; financing and conditions not stated.</t>
+          <t>Conditions unclear: preliminary indication with no stated conditions, though diligence was still open. On time. Pamplona had earlier said its diligence would be minimal.</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a preliminary indication of interest at an all-cash purchase price of $18.50 per share” (p. 33)</t>
+          <t>On July 23, 2013, CSC/Pamplona submitted a preliminary indication of interest at an all-cash purchase price of $18.50 per share. (p. 33)</t>
         </is>
       </c>
       <c r="R21" s="2" t="n"/>
@@ -1847,12 +1846,12 @@
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Preliminary indications due. CSC/Pamplona on time (#20); late: Party B and Party C on 07/24 (#22, #23), Party C written revision 07/25 (#26); all reviewed 07/25. No bids reported from the other 16 signers.</t>
+          <t>Round 1 due date for preliminary indications. CSC/Pamplona bid on time; Party B and Party C bid on 07/24–07/25 and were still considered (late bids accepted).</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>“which they were instructed to submit by July 23, 2013” (p. 32)</t>
+          <t>which they were instructed to submit by July 23, 2013 (p. 32)</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -1877,12 +1876,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>07/24/2013</t>
+          <t>by 07/23/2013</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>16 other financial NDA signers</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1892,7 +1891,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Did not submit</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1901,56 +1900,46 @@
       <c r="G23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: management presentation 08/06; data-room diligence 08/06–08/27. Preliminary indication, one day after the 07/23 due date. Financing not stated.</t>
+          <t>Inferred: 20 signers − Party A (no NDA yet) − 3 submitters = 16; only B, C and CSC/Pamplona indications (plus Party A's 06/21 proposal) were reviewed 07/25. Any member signing after 07/23 would instead have been excluded when four advanced.</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>“Party B submitted a preliminary indication of interest at an all-cash purchase price of $17.00 to $18.00 per share” (p. 33)</t>
+          <t>representatives of BofA Merrill Lynch reviewed the preliminary indications of interest received from Party B, Party C and CSC/Pamplona as well as the Party A June 21 proposal (p. 33)</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="S23" s="2" t="n"/>
       <c r="T23" s="3" t="n">
-        <v>41479</v>
-      </c>
-      <c r="U23" s="3" t="n">
-        <v>41479</v>
-      </c>
+        <v>41478</v>
+      </c>
+      <c r="U23" s="2" t="n"/>
       <c r="V23" s="3" t="n">
-        <v>41479</v>
+        <v>41478</v>
       </c>
     </row>
     <row r="24">
@@ -1964,7 +1953,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>Party B</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1984,10 +1973,10 @@
         <v>1</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -2011,12 +2000,12 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: management presentation 08/08. Oral preliminary indication by phone to BofA, one day after the due date.</t>
+          <t>Conditions unclear: no conditions reported, but diligence was still open. Written preliminary indication one day after the 07/23 due date; reviewed 07/25.</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>“representatives from Party C called BofA Merrill Lynch and presented an oral preliminary indication of interest at an all-cash purchase price of $15.00 to $17.00 per share” (p. 33)</t>
+          <t>On July 24, 2013, Party B submitted a preliminary indication of interest at an all-cash purchase price of $17.00 to $18.00 per share. (p. 33)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -2041,12 +2030,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>by 07/25/2013</t>
+          <t>07/24/2013</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>16 other financial NDA signers</t>
+          <t>Party C</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2056,7 +2045,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -2065,46 +2054,56 @@
       <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
+      <c r="H25" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M25" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Not among the four bidders advanced on 07/25 (#25); no bids from them reported. 20 signers − 4 advanced = 16. Signing dates unknown: any later signer was outside the four-bidder stage (08/27 letters to four only). Q4.</t>
+          <t>Conditions unclear: no conditions reported, diligence still open. Oral preliminary indication made by phone to BofA one day after the due date; reviewed 07/25.</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>“reach out to each of the four interested bidders and arrange management meetings” (p. 34)</t>
+          <t>representatives from Party C called BofA Merrill Lynch and presented an oral preliminary indication of interest at an all-cash purchase price of $15.00 to $17.00 per share (p. 33)</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S25" s="2" t="n"/>
       <c r="T25" s="3" t="n">
-        <v>41480</v>
-      </c>
-      <c r="U25" s="2" t="n"/>
+        <v>41479</v>
+      </c>
+      <c r="U25" s="3" t="n">
+        <v>41479</v>
+      </c>
       <c r="V25" s="3" t="n">
-        <v>41480</v>
+        <v>41479</v>
       </c>
     </row>
     <row r="26">
@@ -2143,12 +2142,12 @@
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Committee found indications low; chose staged disclosure and advanced four: Party A (if it signed a confidentiality agreement), Party B, Party C, CSC/Pamplona, for management meetings (held 08/06–08/14 for all four), then revised indications.</t>
+          <t>Finding the indications lower than expected, the Special Committee advanced four bidders (Party A, if it signed an NDA; B; C; CSC/Pamplona) to management meetings, with staged disclosure of sensitive information, and then revised indications. All four had presentations 08/06–08/14.</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>“authorized and instructed BofA Merrill Lynch to proceed with the staged disclosure as discussed at this meeting and to reach out to each of the four interested bidders” (p. 34)</t>
+          <t>authorized and instructed BofA Merrill Lynch to proceed with the staged disclosure as discussed at this meeting and to reach out to each of the four interested bidders (p. 34)</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -2225,17 +2224,17 @@
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: management presentation 08/08. Written indication after the committee meeting, replacing the oral range (#23): top cut from $17.00 to $16.50.</t>
+          <t>Conditions unclear: no conditions reported, diligence still open. Written indication revising Party C's oral 07/24 range (#24); made after the 07/25 Special Committee meeting and answering the round 1 request.</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>“Party C submitted a written indication of interest at an all-cash purchase price of $16.00 to $16.50 per share” (p. 34)</t>
+          <t>Later on July 25, 2013, Party C submitted a written indication of interest at an all-cash purchase price of $16.00 to $16.50 per share. (p. 34)</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1; Q2</t>
         </is>
       </c>
       <c r="S27" s="2" t="n"/>
@@ -2291,12 +2290,12 @@
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Catch-up access: after talks on non-solicitation terms stalled (07/11–07/23) and resumed 07/27 (filing prints '2103'), Party A signed and got the information package to improve its 06/21 proposal (#8). Already entered at #8.</t>
+          <t>Catch-up access for a late entrant: NDA talks resumed 07/27 once non-solicitation terms were agreed. Party A then received the informational package, to improve its 06/21 proposal. Already live since #7.</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>“Party A entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package” (p. 34)</t>
+          <t>On August 5, 2013, Party A entered into a confidentiality and standstill agreement with Mac-Gray and was provided with an informational package (p. 34)</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -2351,12 +2350,12 @@
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Staged information access: financial bidders Party B and Party C got broad data-room access; strategic bidders Party A and CSC/Pamplona got limited access, customer data incl. locations reserved for later (07/25 staging). Strategics also discussed synergies with management.</t>
+          <t>Information access differed by type: financial bidders B and C got broad data-room access; strategic bidders A and CSC/Pamplona got limited access, with customer data (including locations) held back, but had synergy talks with management.</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>“Party B and Party C, in light of the fact that they were financial bidders, were given broad access to an electronic data site” (p. 34)</t>
+          <t>Party B and Party C, in light of the fact that they were financial bidders, were given broad access to an electronic data site (p. 34)</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -2366,7 +2365,7 @@
       </c>
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="3" t="n">
-        <v>41492</v>
+        <v>41502</v>
       </c>
       <c r="U29" s="3" t="n">
         <v>41492</v>
@@ -2411,17 +2410,17 @@
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>BofA letters to Party A, Party B, Party C and CSC/Pamplona (authorized 08/15): revised written proposals due 09/09/2013 to go on to in-depth evaluation; address valuation, financing, approvals, covenants, diligence focus.</t>
+          <t>BofA's letter to all four bidders set 09/09/2013 as the due date for revised written proposals (valuation, financing, approvals, covenants, diligence), needed to go on to in-depth diligence. Authorized 08/15. Follow-up diligence calls: B 08/27, C 08/29, A 09/03.</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>“instructing such bidders to submit revised written proposals no later than September 9, 2013 if such bidders wished to proceed further in the process” (p. 35)</t>
+          <t>instructing such bidders to submit revised written proposals no later than September 9, 2013 if such bidders wished to proceed further in the process (p. 35)</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S30" s="2" t="n"/>
@@ -2483,7 +2482,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Heavy</t>
         </is>
       </c>
       <c r="M31" s="2" t="n">
@@ -2493,15 +2492,19 @@
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: customer data still reserved; diligence continued 09/11–09/18. Pamplona committed to provide 100% of capital. Requested two-week exclusivity. Revised indication.</t>
+          <t>Heavy: asked for two weeks of exclusive negotiations. Pamplona committed 100% of the required capital. A revised indication, on time; the next stage was to be in-depth diligence.</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a revised indication of interest with an all-cash purchase price of $19.50 per share, indicating that Pamplona was committed to provide 100% of the capital” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R31" s="2" t="n"/>
+          <t>CSC/Pamplona submitted a revised indication of interest with an all-cash purchase price of $19.50 per share, indicating that Pamplona was committed to provide 100% of the capital required (p. 35)</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
       <c r="S31" s="2" t="n"/>
       <c r="T31" s="3" t="n">
         <v>41526</v>
@@ -2571,12 +2574,12 @@
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>No firm financing commitment: to be financed by affiliated-fund equity plus third-party debt (p. 35). Revised indication.</t>
+          <t>Heavy: no firm financing commitment; to be financed by equity from affiliated funds plus third-party debt. A revised indication, on time.</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>“Party B also submitted a revised indication of interest with an all-cash purchase price of $18.50 per share” (p. 35)</t>
+          <t>Party B also submitted a revised indication of interest with an all-cash purchase price of $18.50 per share and proposed to finance the transaction with a combination of equity (p. 35)</t>
         </is>
       </c>
       <c r="R32" s="2" t="n"/>
@@ -2627,17 +2630,17 @@
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>Revised proposals due. CSC/Pamplona and Party B on time (#30, #31); late: Party A and Party C on 09/10 (#33, #34), all reviewed by the committee 09/11.</t>
+          <t>Round 2 due date. CSC/Pamplona and Party B bid on time; Party A and Party C bid on 09/10 and all four were reviewed on 09/11 (late bids accepted).</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>“submit revised written proposals no later than September 9, 2013” (p. 35)</t>
+          <t>submit revised written proposals no later than September 9, 2013 (p. 35)</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S33" s="2" t="n"/>
@@ -2709,17 +2712,17 @@
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>No firm financing commitment (p. 35); to be funded by existing credit facilities or affiliated equity. Revised indication, one day late; floor raised from $17.00 (#8).</t>
+          <t>Heavy: no firm financing commitment (to use outstanding credit facilities or affiliated equity). A revised indication one day after the due date; its range equals its 06/21 proposal (#7).</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>“Party A submitted a revised indication of interest with an all-cash purchase price of $18.00 to $19.00 per share, to be financed by outstanding credit facilities or affiliated equity sources” (p. 35)</t>
+          <t>Party A submitted a revised indication of interest with an all-cash purchase price of $18.00 to $19.00 per share, to be financed by outstanding credit facilities or affiliated equity sources. (p. 35)</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S34" s="2" t="n"/>
@@ -2791,17 +2794,17 @@
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>No firm financing commitment (p. 35). Oral revised indication by phone to BofA, one day late; up from $16.00–16.50 (#26).</t>
+          <t>Heavy: no firm financing commitment. A revised oral indication by phone to BofA, one day after the due date; up from its $16.00–$16.50 written range (#26).</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>“a representative of Party C indicated that it was submitting a revised oral indication of interest with an all-cash purchase price of $16.00 to $17.00 per share” (p. 35)</t>
+          <t>a representative of Party C indicated that it was submitting a revised oral indication of interest with an all-cash purchase price of $16.00 to $17.00 per share (p. 35)</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S35" s="2" t="n"/>
@@ -2826,7 +2829,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Stewart G. MacDonald, Jr. (CEO, large holder)</t>
+          <t>Stewart G. MacDonald, Jr. (CEO and major shareholder)</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
@@ -2851,12 +2854,12 @@
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Rollover refused by holder: MacDonald said he would not roll over shares. BofA reported bidders unlikely to proceed without his express support, so the committee had him fully briefed (09/12); he backed continuing but urged a higher value.</t>
+          <t>Rollover declined: after a limited briefing, MacDonald said he would not roll over any shares. BofA reported that no bidder was likely to proceed without his express support. He was fully briefed on 09/12 and urged seeking a higher value.</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>“Mr. MacDonald indicated that he had decided that he was not interested in rolling over any of his shares in any transaction” (p. 35)</t>
+          <t>Mr. MacDonald indicated that he had decided that he was not interested in rolling over any of his shares in any transaction. (p. 35)</t>
         </is>
       </c>
       <c r="R36" s="2" t="n"/>
@@ -2907,17 +2910,17 @@
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Committee had BofA call all four (Party A, Party B, Party C, CSC/Pamplona) the same day for final indications due 09/18/2013, saying Mac-Gray might grant one bidder short exclusivity depending on price and deal certainty.</t>
+          <t>Special Committee requested final indications from all four bidders by 09/18/2013. BofA told them by phone on 09/11 that Mac-Gray might grant one bidder short exclusivity depending on price and deal certainty. Diligence continued 09/11–09/18.</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>“request final indications of interest by September 18, 2013” (p. 36)</t>
+          <t>the Special Committee instructed BofA Merrill Lynch to call each of Party A, Party B, Party C and CSC/Pamplona to request final indications of interest by September 18, 2013 (p. 36)</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1; Q6; Q7</t>
         </is>
       </c>
       <c r="S37" s="2" t="n"/>
@@ -2979,7 +2982,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Heavy</t>
         </is>
       </c>
       <c r="M38" s="2" t="n">
@@ -2989,17 +2992,17 @@
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: customer data still reserved (#28, #48). Pamplona committed to provide 100% of capital; requested two-week exclusivity. Formal as the answer to the final-indication request, no markup (Q3).</t>
+          <t>Heavy: again asked for two weeks of exclusive negotiations. Pamplona still committed 100% of the capital. Final-round response. Up from $19.50 (#30).</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>“CSC/Pamplona submitted a proposal for an all-cash purchase price of $20.75 per share, reiterating that Pamplona was committed to provide 100% of the capital” (p. 36)</t>
+          <t>CSC/Pamplona submitted a proposal for an all-cash purchase price of $20.75 per share, reiterating that Pamplona was committed to provide 100% of the capital required (p. 36)</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q5; Q7</t>
         </is>
       </c>
       <c r="S38" s="2" t="n"/>
@@ -3034,7 +3037,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Bid reaffirmed</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -3061,7 +3064,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Heavy</t>
         </is>
       </c>
       <c r="M39" s="2" t="n">
@@ -3071,17 +3074,17 @@
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: customer data reserved; diligence continued 09/11–09/18. By price confirmation: Party A told BofA by phone its 09/10 range (#33) was its best and final offer. Financing status at this date not reported.</t>
+          <t>Heavy: repeats its 09/10 indication (#33), which had no firm financing commitment. By phone to BofA, Party A called its $18.00–$19.00 its best and final offer, in response to the final-round request. Price unchanged.</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>“its previous indication of interest with an all-cash purchase price of $18.00 to $19.00 per share was its best and final offer” (p. 36)</t>
+          <t>its previous indication of interest with an all-cash purchase price of $18.00 to $19.00 per share was its best and final offer (p. 36)</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q7</t>
         </is>
       </c>
       <c r="S39" s="2" t="n"/>
@@ -3153,17 +3156,17 @@
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: diligence continued 09/11–09/18. Bidder values offer at $21.50: $19.00 cash at closing plus options on 10% of new equity, vesting on base-case projections over five years, valued by it at $2.50. Committee expected affiliated equity plus third-party debt (p. 37). Q5.</t>
+          <t>Unclear: financing was expected from affiliated-fund equity plus third-party debt, but no commitment status was reported. $19.00 cash at closing plus options on 10% of new equity, vesting on base-case projections over five years; Party B valued the options at $2.50/share.</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>“a revised indication of interest with a purchase price that Party B valued at $21.50 per share, including $19.00 of cash to be paid at closing” (p. 36)</t>
+          <t>Party B also submitted a revised indication of interest with a purchase price that Party B valued at $21.50 per share, including $19.00 of cash to be paid at closing (p. 36)</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
-          <t>Q3; Q5</t>
+          <t>Q7; Q8</t>
         </is>
       </c>
       <c r="S40" s="2" t="n"/>
@@ -3223,12 +3226,12 @@
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Party C neither revised nor reiterated its $16.00–17.00 indication (#34) by the final-indication due date and gave no reason. Its decision.</t>
+          <t>Party C neither submitted a final indication nor reaffirmed its $16.00–$17.00 indication (#34), and gave no reason. Reported 09/19.</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>“Party C did not submit a revised indication of interest or reiterate its prior indication of interest” (p. 36)</t>
+          <t>Party C did not submit a revised indication of interest or reiterate its prior indication of interest of an all-cash purchase price of $16.00 to $17.00 per share (p. 36)</t>
         </is>
       </c>
       <c r="R41" s="2" t="n"/>
@@ -3279,17 +3282,17 @@
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>Final indications due. CSC/Pamplona, Party B and Party A (reaffirmation) answered the same day; Party C did not (#40). Committee chose on the bids in hand on 09/19 (#42).</t>
+          <t>Round 3 due date for final indications. Three bids arrived that day; Party C did not respond. The Special Committee acted on the bids in hand on 09/19.</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>“request final indications of interest by September 18, 2013” (p. 36)</t>
+          <t>request final indications of interest by September 18, 2013 (p. 36)</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="S42" s="2" t="n"/>
@@ -3339,12 +3342,12 @@
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Preferred bidder and price requirement: committee judged CSC/Pamplona best on value, certainty and no third-party financing, despite Party B's higher face value (option risk); offered exclusivity at $21.25. MacDonald said he would support $21.25.</t>
+          <t>Preferred bidder and price requirement: Special Committee judged CSC/Pamplona most valuable and certain (Party B's options risky, its financing riskier) and offered exclusivity at $21.25/share. MacDonald said he would support $21.25.</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>“the Special Committee would be prepared to move into exclusivity at a price of $21.25 per share” (p. 37)</t>
+          <t>authorized the Transaction Committee to inform CSC/Pamplona that the Special Committee would be prepared to move into exclusivity at a price of $21.25 per share (p. 37)</t>
         </is>
       </c>
       <c r="R43" s="2" t="n"/>
@@ -3407,7 +3410,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Heavy</t>
         </is>
       </c>
       <c r="M44" s="2" t="n">
@@ -3417,17 +3420,17 @@
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Diligence open per narrative: customer data not yet released (#48). Pamplona funding 100%, no financing contingency (terms of 09/21–09/23). 'Last and best' answer to #42, conditional on two-week exclusivity; requested MacDonald voting agreements.</t>
+          <t>Heavy: conditioned on two weeks of exclusive negotiations and voting agreements from MacDonald and family. Raised to $21.25 as its last and best offer, the same day the Transaction Committee proposed that price; Pamplona to fund 100%, no financing contingency.</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>“willing to increase their all-cash purchase price to $21.25 per share as a last and best offer, provided that Mac-Gray agree to a two week period of exclusive negotiations” (p. 37)</t>
+          <t>confirm that CSC/Pamplona were willing to increase their all-cash purchase price to $21.25 per share as a last and best offer, provided that Mac-Gray agree to a two week period (p. 37)</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q5; Q7</t>
         </is>
       </c>
       <c r="S44" s="2" t="n"/>
@@ -3447,22 +3450,18 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>09/24/2013</t>
+          <t>09/23/2013</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Mac-Gray and Moab Partners (Rothenberg)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Exclusivity changed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -3476,31 +3475,29 @@
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Executed with CSC and Pamplona to 5 p.m. ET 10/12/2013 (authorized 09/23); lapses if they worsen the final proposal: $21.25 cash, $15m reverse termination fee, no financing contingency, Pamplona funding 100%.</t>
+          <t>Rollover permitted: Goodwin told Rothenberg of the CSC/Pamplona negotiations so that Moab could resume rollover talks with CSC/Pamplona. Rothenberg wanted to, and BofA arranged the talks.</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013” (p. 38)</t>
+          <t>to provide Moab with the opportunity to resume discussions with CSC/Pamplona regarding a possible equity rollover of Moab's shares in the transaction (p. 38)</t>
         </is>
       </c>
       <c r="R45" s="2" t="n"/>
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="3" t="n">
-        <v>41541</v>
+        <v>41540</v>
       </c>
       <c r="U45" s="3" t="n">
-        <v>41541</v>
+        <v>41540</v>
       </c>
       <c r="V45" s="3" t="n">
-        <v>41541</v>
+        <v>41540</v>
       </c>
     </row>
     <row r="46">
@@ -3509,12 +3506,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>by 09/24/2013</t>
+          <t>09/24/2013</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
+          <t>CSC/Pamplona</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3524,7 +3521,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Exclusivity changed</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -3541,24 +3538,16 @@
       <c r="M46" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N46" s="2" t="n"/>
+      <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Inferred: live rival when exclusivity with CSC/Pamplona was executed (#44); filing does not say it was told. Its best and final $18.00–19.00 (#38) was below CSC/Pamplona's $21.25.</t>
+          <t>Executed with CSC/Pamplona until 5 p.m. ET 10/12/2013 (authorized 09/23) on its final proposal: $21.25 cash, $15M reverse termination fee, no financing contingency. Exclusivity lapses automatically if the terms are adversely changed.</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations” (p. 38)</t>
+          <t>CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013 (p. 38)</t>
         </is>
       </c>
       <c r="R46" s="2" t="n"/>
@@ -3567,7 +3556,7 @@
         <v>41541</v>
       </c>
       <c r="U46" s="3" t="n">
-        <v>41535</v>
+        <v>41541</v>
       </c>
       <c r="V46" s="3" t="n">
         <v>41541</v>
@@ -3584,12 +3573,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Party B</t>
+          <t>Party A</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3623,22 +3612,24 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>Inferred: live rival when exclusivity with CSC/Pamplona was executed (#44); not reported as told. Its offer, valued by Party B at $21.50 incl. $19.00 cash (#39), lost on certainty (#42).</t>
+          <t>Inferred: displaced when Mac-Gray signed exclusivity with CSC/Pamplona; the filing never mentions Party A in the process again. Its last offer, $18.00–$19.00, was called best and final (#38).</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations” (p. 38)</t>
-        </is>
-      </c>
-      <c r="R47" s="2" t="n"/>
+          <t>CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013 (p. 38)</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
       <c r="S47" s="2" t="n"/>
       <c r="T47" s="3" t="n">
         <v>41541</v>
       </c>
-      <c r="U47" s="3" t="n">
-        <v>41535</v>
-      </c>
+      <c r="U47" s="2" t="n"/>
       <c r="V47" s="3" t="n">
         <v>41541</v>
       </c>
@@ -3649,18 +3640,22 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>09/25/2013</t>
+          <t>by 09/24/2013</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Kirkland &amp; Ellis LLP</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="n"/>
+          <t>Party B</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -3674,29 +3669,41 @@
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="n"/>
-      <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="n"/>
+      <c r="M48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Outside legal counsel to CSC/Pamplona; first seen acting on 09/25, receiving Goodwin Procter's initial merger-agreement draft.</t>
+          <t>Inferred: displaced by the exclusivity with CSC/Pamplona. On 09/19 the Special Committee preferred CSC/Pamplona over Party B's nominally higher $21.50 package (#39) because of option and financing risk.</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>“Kirkland &amp; Ellis LLP, outside legal counsel to CSC/Pamplona” (p. 38)</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="n"/>
+          <t>CSC, Pamplona and Mac-Gray executed the exclusivity agreement providing for exclusive negotiations until 5 p.m. ET on October 12, 2013 (p. 38)</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="3" t="n">
-        <v>41542</v>
-      </c>
-      <c r="U48" s="3" t="n">
-        <v>41542</v>
-      </c>
+        <v>41541</v>
+      </c>
+      <c r="U48" s="2" t="n"/>
       <c r="V48" s="3" t="n">
-        <v>41542</v>
+        <v>41541</v>
       </c>
     </row>
     <row r="49">
@@ -3705,22 +3712,18 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>between 09/25/2013 and 10/07/2013</t>
+          <t>09/25/2013</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kirkland &amp; Ellis LLP</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Adviser</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -3734,19 +3737,17 @@
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Information access after exclusivity: exclusive bidder CSC/Pamplona granted full data-room access (limited earlier, #28) and management access for confirmatory diligence.</t>
+          <t>Outside legal counsel to CSC/Pamplona; first reported acting when Goodwin sent it the first draft of the merger agreement.</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>“CSC and Pamplona were granted full access to the electronic data site and access to certain members of management and conducted confirmatory business and legal due diligence” (p. 38)</t>
+          <t>Goodwin Procter delivered to Kirkland &amp; Ellis LLP, outside legal counsel to CSC/Pamplona, whom we refer to as Kirkland, the initial draft of the merger agreement (p. 38)</t>
         </is>
       </c>
       <c r="R49" s="2" t="n"/>
@@ -3758,7 +3759,7 @@
         <v>41542</v>
       </c>
       <c r="V49" s="3" t="n">
-        <v>41554</v>
+        <v>41542</v>
       </c>
     </row>
     <row r="50">
@@ -3767,12 +3768,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>between 09/25/2013 and 10/07/2013</t>
+          <t>09/27/2013</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Moab Partners, L.P. (Moab)</t>
+          <t>Stewart G. MacDonald, Jr. and family</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
@@ -3797,24 +3798,24 @@
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Rollover resolved, not formed: after Goodwin told Rothenberg on 09/23 that talks could resume, Moab and Pamplona discussed a rollover and determined none (reported 10/07). Moab signed a voting agreement at signing.</t>
+          <t>Support agreement: MacDonald, his wife and one of his trusts signed voting agreements with CSC/Pamplona (a condition of CSC's 09/21 offer, #43), effective on signing of the merger agreement.</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>“it was determined that Moab would not rollover any Moab shares in the transaction” (p. 38)</t>
+          <t>which were entered into by Mr. MacDonald, his wife and one of his trusts on September 27, 2013, and which became effective upon entry into the merger agreement (p. 39)</t>
         </is>
       </c>
       <c r="R50" s="2" t="n"/>
       <c r="S50" s="2" t="n"/>
       <c r="T50" s="3" t="n">
-        <v>41548</v>
+        <v>41544</v>
       </c>
       <c r="U50" s="3" t="n">
-        <v>41542</v>
+        <v>41544</v>
       </c>
       <c r="V50" s="3" t="n">
-        <v>41554</v>
+        <v>41544</v>
       </c>
     </row>
     <row r="51">
@@ -3823,7 +3824,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>10/12/2013</t>
+          <t>between 09/25/2013 and 10/07/2013</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3838,7 +3839,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Exclusivity changed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -3859,24 +3860,24 @@
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>Extended to 11:59 p.m. ET 10/15/2013 at CSC/Pamplona's request (made by 10/09); committee required a Mac-Gray termination fee of at most $11m, which CSC/Pamplona accepted on 10/11.</t>
+          <t>Information access: in exclusivity, CSC/Pamplona got full data-room access (customer data had been withheld from strategic bidders, #28) and management access, and did confirmatory diligence, including a 10/01 meeting.</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>“CSC, Pamplona and Mac-Gray executed a letter agreement extending exclusivity until 11:59 p.m. ET on October 15, 2013” (p. 41)</t>
+          <t>CSC and Pamplona were granted full access to the electronic data site and access to certain members of management and conducted confirmatory business and legal due diligence (p. 38)</t>
         </is>
       </c>
       <c r="R51" s="2" t="n"/>
       <c r="S51" s="2" t="n"/>
       <c r="T51" s="3" t="n">
-        <v>41559</v>
+        <v>41548</v>
       </c>
       <c r="U51" s="3" t="n">
-        <v>41559</v>
+        <v>41542</v>
       </c>
       <c r="V51" s="3" t="n">
-        <v>41559</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="52">
@@ -3885,22 +3886,18 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>10/14/2013</t>
+          <t>between 09/25/2013 and 10/07/2013</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Moab Partners (Rothenberg)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Merger agreement signed</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -3914,31 +3911,29 @@
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M52" s="2" t="n"/>
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>$21.25 per share in cash; buyers Spin Holdco (Parent), CSC ServiceWorks Holdings and CSC. Pamplona commitment letter $594m; Pamplona liability cap $50m; Mac-Gray fee $11m; CSC reverse fee $15m. Moab and MacDonald voting agreements effective. BofA fairness opinion same day.</t>
+          <t>Rollover abandoned: after talks between Rothenberg and Pamplona, it was decided that Moab would not roll over any shares (reported to the Special Committee 10/07). Moab signed a voting agreement at signing.</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>“Later in the day, on October 14, 2013, the merger agreement was executed, the Pamplona commitment letter was delivered” (p. 41)</t>
+          <t>As a result of such discussions, it was determined that Moab would not rollover any Moab shares in the transaction. (p. 38)</t>
         </is>
       </c>
       <c r="R52" s="2" t="n"/>
       <c r="S52" s="2" t="n"/>
       <c r="T52" s="3" t="n">
-        <v>41561</v>
+        <v>41548</v>
       </c>
       <c r="U52" s="3" t="n">
-        <v>41561</v>
+        <v>41542</v>
       </c>
       <c r="V52" s="3" t="n">
-        <v>41561</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="53">
@@ -3947,60 +3942,184 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>10/15/2013</t>
+          <t>10/12/2013</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="n"/>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Merger announced</t>
+          <t>Exclusivity changed</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
+      <c r="G53" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="n"/>
-      <c r="M53" s="2" t="n"/>
+      <c r="M53" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Joint announcement by Mac-Gray and CSC before the market opened. Ref: $14.72 close 10/11/2013; about 44% premium (p. 5).</t>
+          <t>Extended from 5 p.m. ET 10/12 to 11:59 p.m. ET 10/15/2013 at CSC/Pamplona's request (made 10/09). The Special Committee extended only after CSC/Pamplona accepted an $11M Mac-Gray termination fee on 10/11, down from its proposed $15M.</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>“before the U.S. stock markets opened, Mac-Gray and CSC jointly announced the execution of the merger agreement” (p. 41)</t>
+          <t>On October 12, 2013, CSC, Pamplona and Mac-Gray executed a letter agreement extending exclusivity until 11:59 p.m. ET on October 15, 2013. (p. 41)</t>
         </is>
       </c>
       <c r="R53" s="2" t="n"/>
       <c r="S53" s="2" t="n"/>
       <c r="T53" s="3" t="n">
+        <v>41559</v>
+      </c>
+      <c r="U53" s="3" t="n">
+        <v>41559</v>
+      </c>
+      <c r="V53" s="3" t="n">
+        <v>41559</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>10/14/2013</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>CSC/Pamplona</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Merger agreement signed</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
+      <c r="M54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" s="2" t="n"/>
+      <c r="O54" s="2" t="n"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>$21.25/share cash; Pamplona commitment letter for $594M, no financing condition; $11M target fee; $15M reverse fee; Pamplona damages cap $50M. Moab and MacDonald voting agreements effective. BofA fairness opinion same day.</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>Later in the day, on October 14, 2013, the merger agreement was executed, the Pamplona commitment letter was delivered, Moab and Parent executed the Moab voting agreement (p. 41)</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="n"/>
+      <c r="S54" s="2" t="n"/>
+      <c r="T54" s="3" t="n">
+        <v>41561</v>
+      </c>
+      <c r="U54" s="3" t="n">
+        <v>41561</v>
+      </c>
+      <c r="V54" s="3" t="n">
+        <v>41561</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>10/15/2013</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Mac-Gray and CSC</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Merger announced</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
+      <c r="M55" s="2" t="n"/>
+      <c r="N55" s="2" t="n"/>
+      <c r="O55" s="2" t="n"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Joint announcement before market open. No go-shop, and no competing proposal was reported before the filing (12/04/2013).</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>On October 15, 2013, before the U.S. stock markets opened, Mac-Gray and CSC jointly announced the execution of the merger agreement. (p. 41)</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="n"/>
+      <c r="S55" s="2" t="n"/>
+      <c r="T55" s="3" t="n">
         <v>41562</v>
       </c>
-      <c r="U53" s="3" t="n">
+      <c r="U55" s="3" t="n">
         <v>41562</v>
       </c>
-      <c r="V53" s="3" t="n">
+      <c r="V55" s="3" t="n">
         <v>41562</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V53"/>
+  <autoFilter ref="A1:V55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4018,11 +4137,11 @@
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -4090,12 +4209,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Special Committee's 06/24 decision executed: BofA outreach to 50 parties; confidentiality signers asked for preliminary indications</t>
+          <t>Special Committee decision to approach 50 parties; BofA outreach, NDAs and informational package</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>20 entered: 2 strategic (CSC/Pamplona; Party A via its standing round-0 proposal, no NDA until 08/05) and 18 financial (Party B, Party C, 16 unnamed signers, dates unknown)</t>
+          <t>19 NDA signers furnished the package: 1 strategic (CSC/Pamplona); 18 financial (Party B, Party C, 16 unnamed, some possibly signing after 07/23). Party A (strategic) — 06/21 proposal still being received, not admitted (NDA unsigned until 08/05)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4115,12 +4234,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>3: CSC/Pamplona, Party B, Party C (plus Party A's 06/21 round-0 proposal, reviewed 07/25)</t>
+          <t>3 bidders: CSC/Pamplona (07/23), Party B (07/24), Party C (07/24 oral, 07/25 written); Party A's 06/21 proposal also reviewed</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>four advanced (Party A, Party B, Party C, CSC/Pamplona); 16 other financial signers out</t>
+          <t>four advanced (Party A, Party B, Party C, CSC/Pamplona); 16 financial signers out (inferred Did not submit)</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4255,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>committee advanced four to management meetings and staged diligence, then asked for revised written proposals</t>
+          <t>Special Committee selected four bidders for management meetings and staged diligence, then revised proposals</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4161,12 +4280,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>4: CSC/Pamplona and Party B (09/09), Party A and Party C (09/10)</t>
+          <t>4 bidders: CSC/Pamplona, Party B (09/09); Party A, Party C (09/10)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>all four asked for final indications on 09/11</t>
+          <t>all four asked for final indications; none out</t>
         </is>
       </c>
     </row>
@@ -4182,7 +4301,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>committee asked all four for final indications, holding out short exclusivity</t>
+          <t>BofA called all four bidders requesting final indications of interest</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -4207,12 +4326,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>3: CSC/Pamplona, Party B, Party A (reaffirmed best and final); Party C did not submit</t>
+          <t>3 bidders: CSC/Pamplona, Party A (reiterated best and final), Party B; Party C did not submit</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>CSC/Pamplona selected 09/19 and raised to $21.25 on 09/21; exclusivity 09/24 (Party A, Party B out); signing 10/14</t>
+          <t>CSC/Pamplona preferred 09/19, raised to $21.25 09/21, exclusivity 09/24 (Party A, Party B dropped), signing 10/14/2013</t>
         </is>
       </c>
     </row>
@@ -4228,16 +4347,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4285,27 +4404,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Process and round map: one process with three rounds (outreach 06/24; four advanced 07/25; final indications 09/11)?</t>
+          <t>Process and round map: one process with rounds 0–3?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Yes. One process; round 0 holds Party A's 06/21 proposal; R1 opens with the outreach launched 06/24; R2 on 07/25; R3 on 09/11 (announced final).</t>
+          <t>One process. Round 0: the 04/08 approach to Party A and its 06/21 unsolicited proposal. R1 opens 06/24 (outreach began within four days). R2 opens 07/25 (four selected, management meetings, revised proposals). R3 opens 09/11 (first request for final indications). It ends in exclusivity 09/24 and signing 10/14.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Gaps of two months or more: 04/08/2013 (BofA–Party A call) to 06/21/2013 (Party A proposal), 74 days, both dates certain; no other. C7: (a) fails, since Party A was kept in view (05/09 report; named in 06/24 outreach); (b) fails, gap under three months; (c) met (05/09, 06/24). The 2011–2012 CSC talks had Mac-Gray as buyer (pp. 27–31).</t>
+          <t>Pp. 27–41. Gap of about two months or more with no reported contact with any prospective acquirer: 04/08/2013 to 06/21/2013. E5: (a) fails, since Party A was kept in view; (b) fails, since no end was reported and the gap is under three months; (c) the 06/24 decision is a fresh start. So there is no second process.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>#8, #10, #25, #36, #27, #28</t>
+          <t>#2, #7, #9, #25, #26, #27, #28, #36</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Most plausible alternative: R2 opens with the 08/27 letter, not the 07/25 decision; #25 would move and #27, #28 would fall in R1. R1 opening date alternatives (06/24 decision vs first calls by 06/28) do not move any bid.</t>
+          <t>Plausible alternative: open R2 at the 08/27 due-date letter. Party A's NDA (#27) and the access row (#28) would then move to R1. Party C's 07/25 written bid (#26) stays in R1 either way. Opening R1 on 06/28 (first dated outreach evidence) moves no rows.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -4318,27 +4437,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Deadline outcomes: R1 (07/23) and R2 (09/09) Late bids accepted; R3 (09/18) Enforced?</t>
+          <t>Round 1 deadline outcome (due 07/23/2013)?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Yes. R1: Party B and Party C bid 07/24 (Party C again 07/25) after receiving the 07/23 date, and all were reviewed 07/25. R2: Party A and Party C bid 09/10 and were reviewed 09/11. R3: committee selected CSC/Pamplona 09/19 on the bids in hand.</t>
+          <t>Late bids accepted. CSC/Pamplona bid on 07/23. Party B (written) and Party C (oral) bid on 07/24, and both were reviewed on 07/25; Party C's written 07/25 bid followed. The Deadline set date (06/28, first informational package) is inferred.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Due dates pp. 32, 35, 36; bids pp. 33–36; selection p. 37. The 07/23 instruction went to confidentiality signers, including Party B and Party C, whose agreements predate it (p. 32).</t>
+          <t>P. 32: NDA signers were 'instructed to submit by July 23, 2013'. P. 33: the 07/24 bids, and on 07/25 BofA reviewed the indications from Party B, Party C and CSC/Pamplona.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>#16, #21, #22, #23, #26, #29, #32, #33, #34, #41</t>
+          <t>#13, #21, #23, #24, #26</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>If the one-day slippages were treated as immaterial, R1 and R2 would read Passed without action or Enforced; neither changes any row, but both would overstate enforcement.</t>
+          <t>If 07/23 were treated as a soft target, not a deadline, the outcome becomes Passed without action. Rows and live counts are unchanged.</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -4351,27 +4470,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Are the 09/18 answers to the request for 'final indications of interest' and CSC/Pamplona's 09/21 $21.25 'last and best offer' Formal?</t>
+          <t>Exits and timing of the 16 unnamed financial NDA signers?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Formal (C13 rule 2): the 09/11 request was an announced final solicitation. No markup was delivered; Goodwin sent the first draft only on 09/25. Party A expressly called its range best and final.</t>
+          <t>Keep one cohort: Count 16 on entry (#19) and an inferred Did not submit by 07/23 (#22). No other indications were reported, and only four 'interested bidders' advanced on 07/25.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>The request for final indications came with the prospect of exclusivity (p. 36); CSC/Pamplona called $21.25 its 'last and best offer' (p. 37). Evidence is thin because no documents accompanied the bids.</t>
+          <t>P. 32: 20 signers '(2 strategic, 18 financial)' signed 'over the next two months'. P. 33: only three indications plus Party A's 06/21 proposal were reviewed. P. 34: 'the four interested bidders'.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>#37, #38, #39, #43</t>
+          <t>#19, #22</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>If Informal, the winner reaches signing with no Formal row, and C12 would add a Bid reaffirmed for CSC/Pamplona at 10/07 (Kirkland's revised merger-agreement draft, p. 39), at $21.25 carried from #43, Conditions Unclear.</t>
+          <t>Some of the 16 may have signed after 07/23, some even after 07/25. Those would exit as Dropped by target (07/25 advancement) or Not selected at signing. The Round 1 admitted count would then fall below 19. Total entries are unaffected.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -4384,27 +4503,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The 16 unnamed financial confidentiality signers: are they (and Party B, Party C) within the 35 financial contacts, and did they leave by the 07/25 advancement (Dropped by target) or by the 07/23 due date (Did not submit)?</t>
+          <t>Round 2 deadline outcome (due 09/09/2013)?</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Keep: within the 35; Dropped by target by 07/25, inferred, Count 16.</t>
+          <t>Late bids accepted. CSC/Pamplona and Party B bid on 09/09. Party A and Party C bid on 09/10 and were still reviewed with the others by the Special Committee on 09/11.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The filing gives 20 signers (2 strategic, 18 financial) over two months but no dates for the 16, so it cannot show they had signed before 07/23; the four-bidder set advanced on 07/25 is complete (pp. 32–34).</t>
+          <t>P. 35: the letter required revised proposals 'no later than September 9, 2013'. On 09/10 Party A submitted and Party C gave an oral revised indication. On 09/11 the Committee reviewed the indications of all four.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>#12, #13, #24</t>
+          <t>#29, #32, #33, #34</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Did not submit by 07/23 would change the exit label and round-1 non-submission count, not the live count. If some signed after 07/25, their exit would be by 08/27 (letters to four only).</t>
+          <t>None supported; the two late bids clearly were considered.</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -4417,33 +4536,165 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Party B's 09/18 price: record $21.50 (its own value incl. options) or $19.00 cash?</t>
+          <t>Conditions on CSC/Pamplona's 09/09, 09/18 and 09/21 bids: Heavy or Light?</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>$21.50 in both price cells, All cash = No, with $19.00 cash and $2.50 option value in the Note.</t>
+          <t>Heavy. Each bid asked for, or was conditioned on, a two-week exclusive negotiation period, and E12 counts a stated exclusive period as a further diligence period. The 09/21 bid also required MacDonald voting agreements.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>C15: a stated per-share package value is the total offer value. Party B valued the options at $2.50; the committee questioned that value (pp. 36–37).</t>
+          <t>Pp. 35–37: two weeks of exclusivity was requested on 09/09 and 09/18, and was a proviso of the 09/21 last-and-best offer. Pamplona committed 100% of the capital and had said its diligence would be minimal (p. 32).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>#30, #37, #43</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Light: financing was committed and diligence in exclusivity was only 'confirmatory' (p. 38). Rows #30, #37 and #43 would become Light, making the winner's bids far less conditional than its rivals'.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Round 3 deadline outcome (due 09/18/2013)?</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Enforced. CSC/Pamplona, Party A and Party B responded on 09/18; Party C did not. On 09/19 the Special Committee chose CSC/Pamplona from the bids in hand.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>P. 36: 'request final indications of interest by September 18, 2013'; the 09/18 submissions; and at the 09/19 meeting, 'Party C did not submit'.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>#36, #41</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>None supported.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Is Round 3 a genuine final solicitation, making its bids Formal?</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Yes. Round 3 is Announced as final: BofA asked all four bidders for 'final indications of interest'. The 09/18 responses (#37, #38, #39) and CSC/Pamplona's 09/21 last-and-best offer (#43) are therefore Formal under E11(2). Party A's 09/18 reiteration is a Round 3 Bid, not Bid reaffirmed, because the target was not finalizing with Party A.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>P. 36: 'request final indications of interest by September 18, 2013'. Party A called its range 'best and final'. No markup of the merger agreement was reported before exclusivity; the first draft was sent 09/25 (p. 38).</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>#36, #37, #38, #39, #43</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>If 'final indications' are read as still non-binding, rows #37–#39 and #43 become Informal and the ledger has no Formal bid before signing. Dropping Party A's reiteration row would make it look like a non-response.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>How to price Party B's 09/18 cash-plus-options bid?</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Price cells hold $21.50, Party B's own stated package value: $19.00 cash at closing plus options valued at $2.50. All cash is No. Bid prices are otherwise per-share cash in US dollars.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>P. 36: the purchase price 'that Party B valued at $21.50 per share, including $19.00 of cash'. The options vest on base-case projections over five years. P. 37: the Committee judged them contingent and risky.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>#39</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Using $19.00 would make Party B's final bid lower than CSC/Pamplona's $20.75, changing the reading of why it lost and the ranking of final bids.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Recording $19.00 (cash only) would rank Party B below CSC/Pamplona's $20.75 rather than above it. That changes the interpretation of the winner's selection.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Exit label and reason for Party A and Party B at exclusivity?</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Dropped by target by 09/24 (inferred), when exclusivity with CSC/Pamplona was signed; Exit reason Not stated. The filing never reports either bidder being told it was out, or leaving.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>P. 38: exclusivity executed 09/24. P. 37: on 09/19 the Special Committee preferred CSC/Pamplona on value and certainty. P. 36: Party A called $18–$19 its 'best and final offer'.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>#46, #47</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Party A could take 'Would not improve earlier offer', since it declined to raise its price when asked for final bids. Party B could take 'Lower offer than rivals' on a risk-adjusted view, though it was nominally higher. Either reading changes the valuation information in the exit.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:G10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4457,7 +4708,7 @@
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -4481,7 +4732,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mac-Gray Corporation</t>
+          <t>Mac-Gray Corporation (NYSE), laundry facilities management contractor, Waltham, Massachusetts</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4744,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CSC ServiceWorks, Inc., through Spin Holdco Inc. (Parent), CSC ServiceWorks Holdings, Inc. and CSC Fenway, Inc.; CSC is owned by Pamplona Capital Partners III, L.P., which committed the equity (the filing calls the bidder "CSC/Pamplona")</t>
+          <t>CSC ServiceWorks, Inc., through Spin Holdco Inc. (Parent) and CSC Fenway, Inc. (Merger Subsidiary), with CSC ServiceWorks Holdings, Inc.; CSC is a portfolio company of Pamplona Capital Partners III, L.P., which committed the equity (bidder unit: CSC/Pamplona)</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4756,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Strategic: laundry facilities operator owned by a private equity fund (Pamplona), which funds the deal; the filing calls CSC/Pamplona a strategic bidder (p. 32)</t>
+          <t>Strategic (sponsor-owned operating company; the filing calls CSC/Pamplona a strategic bidder, p. 34)</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4768,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>$21.25 per share in cash; equity funded by a $594m Pamplona commitment letter; no financing condition</t>
+          <t>$21.25 per share in cash; funded by $594 million Pamplona equity commitment, no financing condition (pp. 5–6, 58)</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4816,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>pp. 27–41</t>
+          <t>27–41</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4828,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>target-led: Board authorized BofA to explore opportunities (04/05/2013) and BofA sounded out Party A (04/08); Party A then made an unsolicited proposal (06/21) before the organized outreach. An activist (Moab) won board seats on 05/30/2013 but is not reported pressing for a sale.</t>
+          <t>target-led (board had BofA approach Party A on 04/08/2013 before any bid; Party A's 06/21/2013 proposal was unsolicited; activist Moab won two board seats 05/30/2013 but is not reported pressing for a sale)</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4852,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Winter 2011 into 2012: talks between Mac-Gray and CSC about Mac-Gray acquiring CSC (Mac-Gray as buyer; BofA engaged 10/23/2012); CSC was instead sold to Pamplona in May 2013. Undated discussions with other industry participants. None was a sale of Mac-Gray.</t>
+          <t>Unspecified strategic discussions from time to time with CSC and other industry participants, including 2011–2012 talks about Mac-Gray acquiring CSC (BofA engaged 10/23/2012); CSC was instead sold to Pamplona in May 2013. None was a sale of Mac-Gray (p. 27).</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4864,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Met (process 1): 20 parties. The filing counts 20 potential bidders (parties) signing confidentiality agreements: 2 strategic, 18 financial; CSC and Pamplona counted as one. No post-signing additions.</t>
+          <t>Met (process 1): 20 parties (2 strategic, 18 financial)</t>
         </is>
       </c>
     </row>
@@ -4637,7 +4888,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>US dollars per share. Party B's 09/18 bid mixed $19.00 cash with options it valued at $2.50 per share (Q5); all others all cash.</t>
+          <t>US dollars per share, cash; exception: Party B's 09/18/2013 bid of $19.00 cash plus options it valued at $2.50 (Q8)</t>
         </is>
       </c>
     </row>
@@ -4649,7 +4900,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>BofA Merrill Lynch (Merrill Lynch, Pierce, Fenner &amp; Smith Incorporated), sole financial adviser; engaged 05/31/2013 after its 2011–2012 mandate was ended 05/15/2013</t>
+          <t>BofA Merrill Lynch (Merrill Lynch, Pierce, Fenner &amp; Smith Incorporated)</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4924,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>In spring 2013 Mac-Gray's board, with BofA Merrill Lynch, began exploring a sale; Party A made an unsolicited $17–19 all-cash proposal on 06/21/2013. A Special Committee then had BofA approach 50 parties, and 20 (2 strategic, 18 financial) signed confidentiality agreements. Preliminary indications from CSC/Pamplona ($18.50), Party B ($17–18) and Party C ($15–17, then $16–16.50) led the committee to advance four bidders, including Party A, to management meetings and staged diligence. Revised proposals (09/09–09/10) ranged from $16–17 to $19.50, and final indications on 09/18 brought CSC/Pamplona to $20.75 and Party B to a cash-and-options package it valued at $21.50; Party A stood at $18–19 and Party C dropped out. The committee preferred CSC/Pamplona's fully funded offer, obtained $21.25 in exchange for exclusivity (09/24), and signed on 10/14/2013 after negotiating fees and Pamplona's liability.</t>
+          <t>After Party A signalled interest in April 2013 and made an unsolicited $17–$19 proposal in June, a Special Committee had BofA Merrill Lynch approach 50 parties; 20 signed confidentiality agreements. Three preliminary indications arrived in July, and four bidders (Party A, CSC/Pamplona, and financial bidders Party B and Party C) advanced to management meetings, with customer data withheld from the strategic bidders. Revised indications in September ranged from $16–$17 to $19.50, and a request for final indications drew $20.75 from CSC/Pamplona, a best-and-final $18–$19 from Party A, and a $21.50 cash-and-options package from Party B, while Party C dropped out. The Special Committee preferred CSC/Pamplona's fully equity-backed offer and asked for $21.25, which CSC/Pamplona accepted as its last and best offer in return for two weeks' exclusivity. After exclusivity from 09/24, extended to 10/15, the merger agreement was signed at $21.25 in cash on 10/14/2013 and announced 10/15/2013.</t>
         </is>
       </c>
     </row>

</xml_diff>